<commit_message>
02: situation read revised
</commit_message>
<xml_diff>
--- a/model.xlsx
+++ b/model.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nasir/dev/rizm-fve-takehome-henkel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{234EC3BE-1020-4B4E-9961-FA5F9813FC60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1796F93E-D183-CB42-9000-A95165739CB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21660" activeTab="1" xr2:uid="{D8DCC835-E62D-D344-B61D-C7363F95AE03}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="317">
   <si>
     <t>id</t>
   </si>
@@ -492,9 +492,6 @@
     <t>S7 Annual Report 2025, p. 111</t>
   </si>
   <si>
-    <t>In Düsseldorf, we produce not only laundry detergents and household cleaners but also adhesives for consumers and craftsmen, and products for our industrial customers.</t>
-  </si>
-  <si>
     <t>R22</t>
   </si>
   <si>
@@ -534,9 +531,6 @@
     <t>B</t>
   </si>
   <si>
-    <t>the price a large industrial buyer pays before VAT; band is a guess until the site's purchased volume is known (R30 is the smaller band)</t>
-  </si>
-  <si>
     <t>R29</t>
   </si>
   <si>
@@ -711,9 +705,6 @@
     <t>Plant units in operation: four back-pressure steam turbines</t>
   </si>
   <si>
-    <t>F13G5 20,000 kW gross, 18,000 kW net, commissioned 1980-01-01; F13G6 20,000 / 18,000, 1983-01-01 (also in the BNetzA list, S17); F03G2 13,200 / 11,880, 1965-01-01; F03G3 13,200 / 11,880, 1965-01-01; all natural gas, Gegendruckmaschine mit Entnahme, CHP, in operation, Teileinspeisung</t>
-  </si>
-  <si>
     <t>kW</t>
   </si>
   <si>
@@ -735,9 +726,6 @@
     <t>Plant unit Gasturbine</t>
   </si>
   <si>
-    <t>8,900 kW gross, 8,600 kW net, natural gas, Gasturbine mit Abhitzekessel, CHP, commissioned 2012-02-24, in operation, Teileinspeisung</t>
-  </si>
-  <si>
     <t>S8 Marktstammdatenregister export, KWK933766051545</t>
   </si>
   <si>
@@ -753,9 +741,6 @@
     <t>Plant units retired in 2025</t>
   </si>
   <si>
-    <t>F03G1, 10,000 kW gross, commissioned 1963-01-01, and F12ET, 570 kW, commissioned 1996-01-01, both permanently shut down 2025-07-23</t>
-  </si>
-  <si>
     <t>MaStR unit numbers: SEE956631893736; SEE983086557883; Datum der endgültigen Stilllegung 23.07.2025</t>
   </si>
   <si>
@@ -768,9 +753,6 @@
     <t>Plant as one CHP installation</t>
   </si>
   <si>
-    <t>installation KWK933766051545, commissioned 1948-01-01, elektrische KWK-Leistung 75,300 kW, thermische Nutzleistung 450,000 kW; operator Henkel AG &amp; Co. KGaA (ABR949972975438); grid operator Netzgesellschaft Düsseldorf mbH, Mittelspannung, Teileinspeisung with own consumption; five units in operation, 68,360 kW net (my sum)</t>
-  </si>
-  <si>
     <t>S8 Marktstammdatenregister export</t>
   </si>
   <si>
@@ -813,9 +795,6 @@
     <t>VET 2025 in [t CO2 Äq]: 211.078</t>
   </si>
   <si>
-    <t>whole plant incl. steam and power for third parties; Henkel's own share is not public (third-party share up to 168,856 t per R15), data-request candidate; two small units ran until July 2025 (R47), so 2025 mixes two configurations, effect small; 2024 in R51</t>
-  </si>
-  <si>
     <t>R51</t>
   </si>
   <si>
@@ -825,9 +804,6 @@
     <t>2024 in [t CO2 Äq]: 229.042</t>
   </si>
   <si>
-    <t>D5 sensitivity year; trend 2021: 322,725; 2022: 286,155; 2023: 276,326 (coal exit shows in 2024)</t>
-  </si>
-  <si>
     <t>R52</t>
   </si>
   <si>
@@ -840,24 +816,9 @@
     <t>Zuteilung 2025 in [EUA]: 61.633</t>
   </si>
   <si>
-    <t>allowances to buy = R50 minus R52, priced with R36; 2024: 63,398 EUA</t>
-  </si>
-  <si>
     <t>R53</t>
   </si>
   <si>
-    <t>Group Scope 1 and 2 target and where it stands</t>
-  </si>
-  <si>
-    <t>base year 2021: 778,331; 2025: 392,674 (minus 49.5 % vs base); 2030 target: 451,432 (minus 42 %)</t>
-  </si>
-  <si>
-    <t>Scope 1 and 2 GHG emissions SBTi target scope (t CO2e)1 778,331 461,609 392,674 -14.9% -49.5% 451,432 4.7%</t>
-  </si>
-  <si>
-    <t>the 2030 number is already beaten at group level, so the pressure on the plant comes from the net-zero path and the material-asset finding (R9), not from 2030</t>
-  </si>
-  <si>
     <t>status (opened / not found / irrelevant / not used)</t>
   </si>
   <si>
@@ -991,6 +952,48 @@
   </si>
   <si>
     <t>average German EUA auction price 2025 and 2024</t>
+  </si>
+  <si>
+    <t>Our largest production facilities are located in Bowling Green, Kentucky, USA, and in Düsseldorf, Germany. In Düsseldorf, we produce not only laundry detergents and household cleaners but also adhesives for consumers and craftsmen, and products for our industrial customers.</t>
+  </si>
+  <si>
+    <t>the price a large industrial buyer pays before VAT; band is a guess until the site's purchased volume is known (R30 is the smaller band); a ceiling for a saved kWh, the site imports in some hours and exports in others (R48)</t>
+  </si>
+  <si>
+    <t>F13G5 20 000 kW gross, 18 000 kW net, commissioned 1980-01-01; F13G6 20 000 / 18 000, 1983-01-01 (also in the BNetzA list, S17); F03G2 13 200 / 11 880, 1965-01-01; F03G3 13 200 / 11 880, 1965-01-01; all natural gas, Gegendruckmaschine mit Entnahme, CHP, in operation, Teileinspeisung</t>
+  </si>
+  <si>
+    <t>8 900 kW gross, 8 600 kW net, natural gas, Gasturbine mit Abhitzekessel, CHP, commissioned 2012-02-24, in operation, Teileinspeisung</t>
+  </si>
+  <si>
+    <t>F03G1, 10 000 kW gross, commissioned 1963-01-01, and F12ET, 570 kW, commissioned 1996-01-01, both permanently shut down 2025-07-23</t>
+  </si>
+  <si>
+    <t>installation KWK933766051545, commissioned 1948-01-01, elektrische KWK-Leistung 75 300 kW, thermische Nutzleistung 450 000 kW; operator Henkel AG &amp; Co. KGaA (ABR949972975438); grid operator Netzgesellschaft Düsseldorf mbH, Mittelspannung, Teileinspeisung with own consumption; five units in operation, 68 360 kW net (my sum)</t>
+  </si>
+  <si>
+    <t>whole plant incl. steam and power for third parties; Henkel's own share is not public (third-party share up to 168 856 t per R15), data-request candidate; two small units ran until July 2025 (R47), so 2025 mixes two configurations, effect small; 2024 in R51</t>
+  </si>
+  <si>
+    <t>D5 sensitivity year; trend 2021: 322 725; 2022: 286 155; 2023: 276 326 (coal exit shows in 2024)</t>
+  </si>
+  <si>
+    <t>allowances to buy = R50 minus R52, priced with R36; 2024: 63 398 EUA</t>
+  </si>
+  <si>
+    <t>Group climate targets and where Scope 1 and 2 stand</t>
+  </si>
+  <si>
+    <t>base year 2021: 778,331; 2025: 392,674 (minus 49.5 % vs base); 2030 target 1: 451,432 (minus 42 %, Scope 1 and 2 combined); target 3 net zero: minus 90 % across Scopes 1, 2 and 3 by 2045</t>
+  </si>
+  <si>
+    <t>S7 Annual Report 2025, pp. 200 and 205</t>
+  </si>
+  <si>
+    <t>Scope 1 and 2 GHG emissions SBTi target scope (t CO2e)1 778,331 461,609 392,674 -14.9% -49.5% 451,432 4.7% | p. 200: Our target 1: Reduce absolute Scope 1 and 2 GHG emissions by 42% (2030 vs. 2021). Our target 3 (net zero): Reduce absolute Scope 1, Scope 2 and Scope 3 GHG emissions by 90% (2045 vs 2021)</t>
+  </si>
+  <si>
+    <t>hand check: R53 = R15 gross Scope 1 + R17 market-based Scope 2 for 2021 and 2025; the combined KPI is past minus 42 % because market-based Scope 2 fell from 160 242 to 34 824; Scope 1 alone is 357 850 vs 618 089 = minus 42.1 %, on the 2030 line; with Scope 2 nearly used up, Scope 1 is the remaining lever toward 2045 (my inference, target 3 is combined across all scopes); no Scope 1-only target exists, the p. 203 sentence in R9 refers to the plant's share of target 1</t>
   </si>
 </sst>
 </file>
@@ -1390,7 +1393,7 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>271</v>
+        <v>258</v>
       </c>
       <c r="E1" t="s">
         <v>3</v>
@@ -1476,7 +1479,7 @@
         <v>46290</v>
       </c>
       <c r="F5" t="s">
-        <v>272</v>
+        <v>259</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -1501,10 +1504,10 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>273</v>
+        <v>260</v>
       </c>
       <c r="B7" t="s">
-        <v>274</v>
+        <v>261</v>
       </c>
       <c r="C7" t="s">
         <v>81</v>
@@ -1516,15 +1519,15 @@
         <v>46290</v>
       </c>
       <c r="F7" t="s">
-        <v>275</v>
+        <v>262</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>276</v>
+        <v>263</v>
       </c>
       <c r="B8" t="s">
-        <v>277</v>
+        <v>264</v>
       </c>
       <c r="C8" t="s">
         <v>89</v>
@@ -1536,18 +1539,18 @@
         <v>46290</v>
       </c>
       <c r="F8" t="s">
-        <v>278</v>
+        <v>265</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>279</v>
+        <v>266</v>
       </c>
       <c r="B9" t="s">
-        <v>280</v>
+        <v>267</v>
       </c>
       <c r="C9" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="D9" t="s">
         <v>41</v>
@@ -1556,18 +1559,18 @@
         <v>46290</v>
       </c>
       <c r="F9" t="s">
-        <v>281</v>
+        <v>268</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>282</v>
+        <v>269</v>
       </c>
       <c r="B10" t="s">
-        <v>283</v>
+        <v>270</v>
       </c>
       <c r="C10" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D10" t="s">
         <v>41</v>
@@ -1576,18 +1579,18 @@
         <v>46290</v>
       </c>
       <c r="F10" t="s">
-        <v>284</v>
+        <v>271</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>285</v>
+        <v>272</v>
       </c>
       <c r="B11" t="s">
-        <v>286</v>
+        <v>273</v>
       </c>
       <c r="C11" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D11" t="s">
         <v>41</v>
@@ -1596,18 +1599,18 @@
         <v>46290</v>
       </c>
       <c r="F11" t="s">
-        <v>287</v>
+        <v>274</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>288</v>
+        <v>275</v>
       </c>
       <c r="B12" t="s">
-        <v>289</v>
+        <v>276</v>
       </c>
       <c r="C12" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="D12" t="s">
         <v>41</v>
@@ -1616,38 +1619,38 @@
         <v>46290</v>
       </c>
       <c r="F12" t="s">
-        <v>290</v>
+        <v>277</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>291</v>
+        <v>278</v>
       </c>
       <c r="B13" t="s">
-        <v>292</v>
+        <v>279</v>
       </c>
       <c r="C13" t="s">
-        <v>293</v>
+        <v>280</v>
       </c>
       <c r="D13" t="s">
-        <v>294</v>
+        <v>281</v>
       </c>
       <c r="E13" s="1">
         <v>46290</v>
       </c>
       <c r="F13" t="s">
-        <v>295</v>
+        <v>282</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>296</v>
+        <v>283</v>
       </c>
       <c r="B14" t="s">
-        <v>297</v>
+        <v>284</v>
       </c>
       <c r="C14" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="D14" t="s">
         <v>41</v>
@@ -1656,38 +1659,38 @@
         <v>46290</v>
       </c>
       <c r="F14" t="s">
-        <v>298</v>
+        <v>285</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>299</v>
+        <v>286</v>
       </c>
       <c r="B15" t="s">
-        <v>300</v>
+        <v>287</v>
       </c>
       <c r="C15" t="s">
-        <v>301</v>
+        <v>288</v>
       </c>
       <c r="D15" t="s">
-        <v>294</v>
+        <v>281</v>
       </c>
       <c r="E15" s="1">
         <v>46290</v>
       </c>
       <c r="F15" t="s">
-        <v>302</v>
+        <v>289</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>303</v>
+        <v>290</v>
       </c>
       <c r="B16" t="s">
-        <v>304</v>
+        <v>291</v>
       </c>
       <c r="C16" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="D16" t="s">
         <v>41</v>
@@ -1696,18 +1699,18 @@
         <v>46290</v>
       </c>
       <c r="F16" t="s">
-        <v>305</v>
+        <v>292</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>306</v>
+        <v>293</v>
       </c>
       <c r="B17" t="s">
-        <v>307</v>
+        <v>294</v>
       </c>
       <c r="C17" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="D17" t="s">
         <v>41</v>
@@ -1716,18 +1719,18 @@
         <v>46290</v>
       </c>
       <c r="F17" t="s">
-        <v>308</v>
+        <v>295</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>309</v>
+        <v>296</v>
       </c>
       <c r="B18" t="s">
-        <v>310</v>
+        <v>297</v>
       </c>
       <c r="C18" t="s">
-        <v>311</v>
+        <v>298</v>
       </c>
       <c r="D18" t="s">
         <v>41</v>
@@ -1736,18 +1739,18 @@
         <v>46290</v>
       </c>
       <c r="F18" t="s">
-        <v>312</v>
+        <v>299</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>313</v>
+        <v>300</v>
       </c>
       <c r="B19" t="s">
-        <v>314</v>
+        <v>301</v>
       </c>
       <c r="C19" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D19" t="s">
         <v>41</v>
@@ -1756,7 +1759,7 @@
         <v>46290</v>
       </c>
       <c r="F19" t="s">
-        <v>315</v>
+        <v>302</v>
       </c>
     </row>
   </sheetData>
@@ -2451,7 +2454,7 @@
         <v>89</v>
       </c>
       <c r="I17" t="s">
-        <v>149</v>
+        <v>303</v>
       </c>
       <c r="J17">
         <v>2025</v>
@@ -2468,13 +2471,13 @@
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
+        <v>149</v>
+      </c>
+      <c r="B18" t="s">
         <v>150</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
         <v>151</v>
-      </c>
-      <c r="C18" t="s">
-        <v>152</v>
       </c>
       <c r="D18" t="s">
         <v>58</v>
@@ -2489,7 +2492,7 @@
         <v>89</v>
       </c>
       <c r="I18" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="J18">
         <v>2025</v>
@@ -2504,33 +2507,33 @@
         <v>46290</v>
       </c>
       <c r="O18" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
+        <v>154</v>
+      </c>
+      <c r="B19" t="s">
         <v>155</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19" t="s">
         <v>156</v>
-      </c>
-      <c r="C19" t="s">
-        <v>157</v>
       </c>
       <c r="D19" t="s">
         <v>58</v>
       </c>
       <c r="E19" t="s">
+        <v>157</v>
+      </c>
+      <c r="G19" t="s">
         <v>158</v>
       </c>
-      <c r="G19" t="s">
+      <c r="H19" t="s">
         <v>159</v>
       </c>
-      <c r="H19" t="s">
+      <c r="I19" t="s">
         <v>160</v>
-      </c>
-      <c r="I19" t="s">
-        <v>161</v>
       </c>
       <c r="J19">
         <v>2025</v>
@@ -2539,39 +2542,39 @@
         <v>61</v>
       </c>
       <c r="L19" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M19" s="1">
         <v>46290</v>
       </c>
       <c r="O19" t="s">
-        <v>163</v>
+        <v>304</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
+        <v>162</v>
+      </c>
+      <c r="B20" t="s">
+        <v>163</v>
+      </c>
+      <c r="C20" t="s">
         <v>164</v>
-      </c>
-      <c r="B20" t="s">
-        <v>165</v>
-      </c>
-      <c r="C20" t="s">
-        <v>166</v>
       </c>
       <c r="D20" t="s">
         <v>58</v>
       </c>
       <c r="E20" t="s">
+        <v>157</v>
+      </c>
+      <c r="G20" t="s">
         <v>158</v>
       </c>
-      <c r="G20" t="s">
+      <c r="H20" t="s">
         <v>159</v>
       </c>
-      <c r="H20" t="s">
-        <v>160</v>
-      </c>
       <c r="I20" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="J20">
         <v>2024</v>
@@ -2580,39 +2583,39 @@
         <v>61</v>
       </c>
       <c r="L20" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M20" s="1">
         <v>46290</v>
       </c>
       <c r="O20" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
+        <v>167</v>
+      </c>
+      <c r="B21" t="s">
+        <v>168</v>
+      </c>
+      <c r="C21" t="s">
         <v>169</v>
-      </c>
-      <c r="B21" t="s">
-        <v>170</v>
-      </c>
-      <c r="C21" t="s">
-        <v>171</v>
       </c>
       <c r="D21" t="s">
         <v>58</v>
       </c>
       <c r="E21" t="s">
+        <v>157</v>
+      </c>
+      <c r="G21" t="s">
         <v>158</v>
       </c>
-      <c r="G21" t="s">
+      <c r="H21" t="s">
         <v>159</v>
       </c>
-      <c r="H21" t="s">
-        <v>160</v>
-      </c>
       <c r="I21" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="J21">
         <v>2025</v>
@@ -2621,39 +2624,39 @@
         <v>61</v>
       </c>
       <c r="L21" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M21" s="1">
         <v>46290</v>
       </c>
       <c r="O21" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
+        <v>172</v>
+      </c>
+      <c r="B22" t="s">
+        <v>173</v>
+      </c>
+      <c r="C22" t="s">
         <v>174</v>
-      </c>
-      <c r="B22" t="s">
-        <v>175</v>
-      </c>
-      <c r="C22" t="s">
-        <v>176</v>
       </c>
       <c r="D22" t="s">
         <v>58</v>
       </c>
       <c r="E22" t="s">
+        <v>175</v>
+      </c>
+      <c r="G22" t="s">
+        <v>176</v>
+      </c>
+      <c r="H22" t="s">
         <v>177</v>
       </c>
-      <c r="G22" t="s">
+      <c r="I22" t="s">
         <v>178</v>
-      </c>
-      <c r="H22" t="s">
-        <v>179</v>
-      </c>
-      <c r="I22" t="s">
-        <v>180</v>
       </c>
       <c r="J22">
         <v>2025</v>
@@ -2662,39 +2665,39 @@
         <v>61</v>
       </c>
       <c r="L22" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M22" s="1">
         <v>46290</v>
       </c>
       <c r="O22" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
+        <v>180</v>
+      </c>
+      <c r="B23" t="s">
+        <v>181</v>
+      </c>
+      <c r="C23" t="s">
         <v>182</v>
-      </c>
-      <c r="B23" t="s">
-        <v>183</v>
-      </c>
-      <c r="C23" t="s">
-        <v>184</v>
       </c>
       <c r="D23" t="s">
         <v>58</v>
       </c>
       <c r="E23" t="s">
+        <v>175</v>
+      </c>
+      <c r="G23" t="s">
+        <v>176</v>
+      </c>
+      <c r="H23" t="s">
         <v>177</v>
       </c>
-      <c r="G23" t="s">
-        <v>178</v>
-      </c>
-      <c r="H23" t="s">
-        <v>179</v>
-      </c>
       <c r="I23" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="J23">
         <v>2024</v>
@@ -2703,21 +2706,21 @@
         <v>61</v>
       </c>
       <c r="L23" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M23" s="1">
         <v>46290</v>
       </c>
       <c r="O23" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B24" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C24">
         <v>65</v>
@@ -2726,16 +2729,16 @@
         <v>58</v>
       </c>
       <c r="E24" t="s">
+        <v>186</v>
+      </c>
+      <c r="G24" t="s">
+        <v>187</v>
+      </c>
+      <c r="H24" t="s">
         <v>188</v>
       </c>
-      <c r="G24" t="s">
+      <c r="I24" t="s">
         <v>189</v>
-      </c>
-      <c r="H24" t="s">
-        <v>190</v>
-      </c>
-      <c r="I24" t="s">
-        <v>191</v>
       </c>
       <c r="J24">
         <v>2024</v>
@@ -2744,42 +2747,42 @@
         <v>61</v>
       </c>
       <c r="L24" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M24" s="1">
         <v>46290</v>
       </c>
       <c r="O24" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
+        <v>191</v>
+      </c>
+      <c r="B25" t="s">
+        <v>192</v>
+      </c>
+      <c r="C25" t="s">
         <v>193</v>
-      </c>
-      <c r="B25" t="s">
-        <v>194</v>
-      </c>
-      <c r="C25" t="s">
-        <v>195</v>
       </c>
       <c r="D25">
         <v>74</v>
       </c>
       <c r="E25" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="F25" t="s">
+        <v>194</v>
+      </c>
+      <c r="G25" t="s">
+        <v>195</v>
+      </c>
+      <c r="H25" t="s">
         <v>196</v>
       </c>
-      <c r="G25" t="s">
+      <c r="I25" t="s">
         <v>197</v>
-      </c>
-      <c r="H25" t="s">
-        <v>198</v>
-      </c>
-      <c r="I25" t="s">
-        <v>199</v>
       </c>
       <c r="J25">
         <v>2025</v>
@@ -2794,15 +2797,15 @@
         <v>46290</v>
       </c>
       <c r="O25" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="B26" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C26">
         <v>89</v>
@@ -2811,16 +2814,16 @@
         <v>58</v>
       </c>
       <c r="E26" t="s">
+        <v>201</v>
+      </c>
+      <c r="G26" t="s">
+        <v>202</v>
+      </c>
+      <c r="H26" t="s">
         <v>203</v>
       </c>
-      <c r="G26" t="s">
+      <c r="I26" t="s">
         <v>204</v>
-      </c>
-      <c r="H26" t="s">
-        <v>205</v>
-      </c>
-      <c r="I26" t="s">
-        <v>206</v>
       </c>
       <c r="J26">
         <v>2023</v>
@@ -2829,21 +2832,21 @@
         <v>83</v>
       </c>
       <c r="L26" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M26" s="1">
         <v>46290</v>
       </c>
       <c r="O26" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B27" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="C27">
         <v>85</v>
@@ -2855,13 +2858,13 @@
         <v>120</v>
       </c>
       <c r="G27" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="H27" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="I27" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="J27">
         <v>2023</v>
@@ -2870,24 +2873,24 @@
         <v>83</v>
       </c>
       <c r="L27" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M27" s="1">
         <v>46290</v>
       </c>
       <c r="O27" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
+        <v>211</v>
+      </c>
+      <c r="B28" t="s">
+        <v>212</v>
+      </c>
+      <c r="C28" t="s">
         <v>213</v>
-      </c>
-      <c r="B28" t="s">
-        <v>214</v>
-      </c>
-      <c r="C28" t="s">
-        <v>215</v>
       </c>
       <c r="D28" t="s">
         <v>58</v>
@@ -2896,13 +2899,13 @@
         <v>59</v>
       </c>
       <c r="G28" t="s">
+        <v>214</v>
+      </c>
+      <c r="H28" t="s">
+        <v>215</v>
+      </c>
+      <c r="I28" t="s">
         <v>216</v>
-      </c>
-      <c r="H28" t="s">
-        <v>217</v>
-      </c>
-      <c r="I28" t="s">
-        <v>218</v>
       </c>
       <c r="J28">
         <v>2014</v>
@@ -2911,39 +2914,39 @@
         <v>83</v>
       </c>
       <c r="L28" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M28" s="1">
         <v>46290</v>
       </c>
       <c r="O28" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B29" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C29" t="s">
-        <v>222</v>
+        <v>305</v>
       </c>
       <c r="D29" t="s">
         <v>58</v>
       </c>
       <c r="E29" t="s">
+        <v>220</v>
+      </c>
+      <c r="G29" t="s">
+        <v>221</v>
+      </c>
+      <c r="H29" t="s">
+        <v>222</v>
+      </c>
+      <c r="I29" t="s">
         <v>223</v>
-      </c>
-      <c r="G29" t="s">
-        <v>224</v>
-      </c>
-      <c r="H29" t="s">
-        <v>225</v>
-      </c>
-      <c r="I29" t="s">
-        <v>226</v>
       </c>
       <c r="J29">
         <v>2026</v>
@@ -2958,33 +2961,33 @@
         <v>46290</v>
       </c>
       <c r="O29" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="B30" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="C30" t="s">
-        <v>230</v>
+        <v>306</v>
       </c>
       <c r="D30" t="s">
         <v>58</v>
       </c>
       <c r="E30" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="G30" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="H30" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="I30" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="J30">
         <v>2026</v>
@@ -2999,33 +3002,33 @@
         <v>46290</v>
       </c>
       <c r="O30" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="B31" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="C31" t="s">
-        <v>236</v>
+        <v>307</v>
       </c>
       <c r="D31" t="s">
         <v>58</v>
       </c>
       <c r="E31" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="G31" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="H31" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="I31" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="J31">
         <v>2025</v>
@@ -3040,33 +3043,33 @@
         <v>46290</v>
       </c>
       <c r="O31" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="B32" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="C32" t="s">
-        <v>241</v>
+        <v>308</v>
       </c>
       <c r="D32" t="s">
         <v>58</v>
       </c>
       <c r="E32" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="G32" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="H32" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="I32" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="J32">
         <v>2026</v>
@@ -3081,18 +3084,18 @@
         <v>46290</v>
       </c>
       <c r="O32" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="B33" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
       <c r="C33" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="D33" t="s">
         <v>58</v>
@@ -3101,13 +3104,13 @@
         <v>59</v>
       </c>
       <c r="G33" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="H33" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="I33" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="J33">
         <v>2025</v>
@@ -3122,15 +3125,15 @@
         <v>46290</v>
       </c>
       <c r="O33" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="B34" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="C34">
         <v>211.078</v>
@@ -3139,16 +3142,16 @@
         <v>211078</v>
       </c>
       <c r="E34" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="G34" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="H34" t="s">
+        <v>243</v>
+      </c>
+      <c r="I34" t="s">
         <v>249</v>
-      </c>
-      <c r="I34" t="s">
-        <v>255</v>
       </c>
       <c r="J34">
         <v>2025</v>
@@ -3163,15 +3166,15 @@
         <v>46290</v>
       </c>
       <c r="O34" t="s">
-        <v>256</v>
+        <v>309</v>
       </c>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="B35" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
       <c r="C35">
         <v>229.042</v>
@@ -3180,16 +3183,16 @@
         <v>229042</v>
       </c>
       <c r="E35" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="G35" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="H35" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="I35" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="J35">
         <v>2024</v>
@@ -3204,15 +3207,15 @@
         <v>46290</v>
       </c>
       <c r="O35" t="s">
-        <v>260</v>
+        <v>310</v>
       </c>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>261</v>
+        <v>253</v>
       </c>
       <c r="B36" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="C36">
         <v>61.633000000000003</v>
@@ -3221,16 +3224,16 @@
         <v>61633</v>
       </c>
       <c r="E36" t="s">
-        <v>263</v>
+        <v>255</v>
       </c>
       <c r="G36" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="H36" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="I36" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
       <c r="J36">
         <v>2025</v>
@@ -3245,18 +3248,18 @@
         <v>46290</v>
       </c>
       <c r="O36" t="s">
-        <v>265</v>
+        <v>311</v>
       </c>
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="B37" t="s">
-        <v>267</v>
+        <v>312</v>
       </c>
       <c r="C37" t="s">
-        <v>268</v>
+        <v>313</v>
       </c>
       <c r="D37" t="s">
         <v>58</v>
@@ -3265,13 +3268,13 @@
         <v>113</v>
       </c>
       <c r="G37" t="s">
-        <v>114</v>
+        <v>314</v>
       </c>
       <c r="H37" t="s">
         <v>89</v>
       </c>
       <c r="I37" t="s">
-        <v>269</v>
+        <v>315</v>
       </c>
       <c r="J37">
         <v>2025</v>
@@ -3286,7 +3289,7 @@
         <v>46290</v>
       </c>
       <c r="O37" t="s">
-        <v>270</v>
+        <v>316</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
03: longlist, ranking, cut decisions
</commit_message>
<xml_diff>
--- a/model.xlsx
+++ b/model.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nasir/dev/rizm-fve-takehome-henkel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1796F93E-D183-CB42-9000-A95165739CB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20B0C9BB-5F45-264B-B849-5E2581413CED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21660" activeTab="1" xr2:uid="{D8DCC835-E62D-D344-B61D-C7363F95AE03}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21660" activeTab="2" xr2:uid="{D8DCC835-E62D-D344-B61D-C7363F95AE03}"/>
   </bookViews>
   <sheets>
     <sheet name="sources" sheetId="4" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="calc" sheetId="5" r:id="rId4"/>
     <sheet name="hand_check" sheetId="3" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="317">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="416">
   <si>
     <t>id</t>
   </si>
@@ -129,12 +129,6 @@
     <t>rank</t>
   </si>
   <si>
-    <t>status (shortlist / cut)</t>
-  </si>
-  <si>
-    <t>cut_reason</t>
-  </si>
-  <si>
     <t>S1</t>
   </si>
   <si>
@@ -582,9 +576,6 @@
     <t>Band I5: 1 000 000 GJ &lt; consumption &lt; 4 000 000 GJ; Excluding taxes and levies; 2025-S1 0.0422, 2025-S2 0.0353</t>
   </si>
   <si>
-    <t>right basis for an ETS plant: no BEHG levy; energy tax on CHP fuel is largely refunded (my knowledge, not sourced); band fits: R50 at the standard gas factor (56.1 t CO2 per TJ) implies roughly 3.8 million GJ a year, my estimate</t>
-  </si>
-  <si>
     <t>R32</t>
   </si>
   <si>
@@ -994,6 +985,312 @@
   </si>
   <si>
     <t>hand check: R53 = R15 gross Scope 1 + R17 market-based Scope 2 for 2021 and 2025; the combined KPI is past minus 42 % because market-based Scope 2 fell from 160 242 to 34 824; Scope 1 alone is 357 850 vs 618 089 = minus 42.1 %, on the 2030 line; with Scope 2 nearly used up, Scope 1 is the remaining lever toward 2045 (my inference, target 3 is combined across all scopes); no Scope 1-only target exists, the p. 203 sentence in R9 refers to the plant's share of target 1</t>
+  </si>
+  <si>
+    <t>reason</t>
+  </si>
+  <si>
+    <t>R42, R46, R48, R8, R5, R1</t>
+  </si>
+  <si>
+    <t>15-min steam and electricity meters per consumer, unit heat rates, start costs, minimum loads</t>
+  </si>
+  <si>
+    <t>Third-party steam may be fixed-schedule under contract [guess]; forecast value small if load is already flat</t>
+  </si>
+  <si>
+    <t>Gas turbine dispatch on day-ahead/intraday spread (spark spread incl. EUA)</t>
+  </si>
+  <si>
+    <t>R46, R1, R31, R36, R28, R48</t>
+  </si>
+  <si>
+    <t>GT heat rate and Abhitzekessel heat credit, hourly spot prices, gas contract price, export tariff, ramp/start limits</t>
+  </si>
+  <si>
+    <t>8.6 MW net is small [found R46]; GT heat may be needed for district heating since April 2026 [inferred from R8]</t>
+  </si>
+  <si>
+    <t>Import/export optimisation at the medium-voltage connection incl. network-charge rules (peak, atypical use)</t>
+  </si>
+  <si>
+    <t>R48, R28, R30, R1, R3</t>
+  </si>
+  <si>
+    <t>15-min import/export, grid contract and tariff, peak billing basis, KWKG/feed-in terms</t>
+  </si>
+  <si>
+    <t>Site may be net exporter most hours [guess]; feed-in terms may be fixed [assumes: no fixed-price feed-in contract]</t>
+  </si>
+  <si>
+    <t>U4</t>
+  </si>
+  <si>
+    <t>Gas, power and EUA hedging to a risk tolerance (futures, PPA, EUA position)</t>
+  </si>
+  <si>
+    <t>R3, R2, R31, R32, R35, R36, R50, R52, R11</t>
+  </si>
+  <si>
+    <t>Annual gas volume, hedge ratio and timing, EUA position, purchased-power volume, risk appetite</t>
+  </si>
+  <si>
+    <t>Group treasury may already hedge centrally [guess]; [assumes: site or Henkel DE procures its own gas and EUAs]</t>
+  </si>
+  <si>
+    <t>U5</t>
+  </si>
+  <si>
+    <t>Shifting electricity-intensive process steps into cheap/green hours</t>
+  </si>
+  <si>
+    <t>R4, R20, R28, R1</t>
+  </si>
+  <si>
+    <t>Load profiles per line, batch/campaign constraints, buffer sizes, staffing rules</t>
+  </si>
+  <si>
+    <t>Own CHP power dampens the spot signal [inferred from R48]; detergent/adhesive lines may be continuous or quality-bound [guess]; [assumes: shiftable electric loads exist]</t>
+  </si>
+  <si>
+    <t>U6</t>
+  </si>
+  <si>
+    <t>Control-reserve and intraday flexibility from GT and steam-turbine extraction</t>
+  </si>
+  <si>
+    <t>R1, R46, R42, R48</t>
+  </si>
+  <si>
+    <t>Ramp rates, prequalification status, controllable MW, steam-extraction limits, aggregator terms</t>
+  </si>
+  <si>
+    <t>Back-pressure units cannot vary power without varying steam [inferred from R42]; [assumes: no existing prequalification]</t>
+  </si>
+  <si>
+    <t>U7</t>
+  </si>
+  <si>
+    <t>Biomethane volume and timing against EUA price, gas price and 2030 Scope 1 path</t>
+  </si>
+  <si>
+    <t>R10, R9, R36, R50, R52, R53, R14</t>
+  </si>
+  <si>
+    <t>Biomethane offer prices, sustainability certification, ETS zero-rating conditions, target trajectory per year</t>
+  </si>
+  <si>
+    <t>[already done: started per R10]; mass-balance biomethane may not zero-rate under ETS without certification [guess]</t>
+  </si>
+  <si>
+    <t>U8</t>
+  </si>
+  <si>
+    <t>Investment case: electrode boiler, industrial heat pump or steam storage beside the CHP</t>
+  </si>
+  <si>
+    <t>R2, R42, R48, R38, R28, R31, R36, R50</t>
+  </si>
+  <si>
+    <t>Steam pressure/temperature levels, load-duration curve, hourly power prices, CAPEX quotes, grid capacity</t>
+  </si>
+  <si>
+    <t>85 % CHP efficiency [found R38] and 13 ct vs 4 ct price gap [inferred from R28, R31] make electrification hard; [assumes: low-pressure steam share large enough]</t>
+  </si>
+  <si>
+    <t>U9</t>
+  </si>
+  <si>
+    <t>Heat source split for district-heating deliveries (waste heat vs CHP heat)</t>
+  </si>
+  <si>
+    <t>R8, R10, R42, R46</t>
+  </si>
+  <si>
+    <t>Heat contract volumes and prices, waste-heat availability per hour, CHP heat cost</t>
+  </si>
+  <si>
+    <t>[already done: sale itself]; contract may be take-or-pay with no dispatch freedom [guess]</t>
+  </si>
+  <si>
+    <t>U10</t>
+  </si>
+  <si>
+    <t>Third-party steam and power cost allocation at 15-min resolution (BASF, KLK)</t>
+  </si>
+  <si>
+    <t>R3, R15, R49, R48</t>
+  </si>
+  <si>
+    <t>Steam/power meters per tenant, contract pricing formulas, plant marginal cost per hour</t>
+  </si>
+  <si>
+    <t>Pass-through contracts yield no € for Henkel [guess]; [assumes: BASF and KLK are the steam customers, inferred from R49]</t>
+  </si>
+  <si>
+    <t>U11</t>
+  </si>
+  <si>
+    <t>Boiler and turbine efficiency monitoring (flue gas, condensate return, fouling)</t>
+  </si>
+  <si>
+    <t>R10, R38, R42, R22</t>
+  </si>
+  <si>
+    <t>Boiler-level fuel and steam meters, flue-gas O2/temperature, condensate return rate</t>
+  </si>
+  <si>
+    <t>[already done: "efficiency" is in Henkel's plan per R10]; needs meter granularity that may not exist [guess]</t>
+  </si>
+  <si>
+    <t>U12</t>
+  </si>
+  <si>
+    <t>U13</t>
+  </si>
+  <si>
+    <t>(forecasting) Fewer boiler/turbine starts and less steam venting per ton of product, because four units follow steam [inferred from R42]</t>
+  </si>
+  <si>
+    <t>(operations) Runs the one steam-independent unit only in hours where power value exceeds gas + CO2 cost [inferred from R46, R31, R36]</t>
+  </si>
+  <si>
+    <t>(procurement and trading) Cuts purchased kWh at ~13 ct and peak charges, values exports in high-price hours [inferred from R28, R48]</t>
+  </si>
+  <si>
+    <t>(procurement and trading) Lowers average €/MWh gas and €/EUA paid for the ~150 kt of allowances bought each year [inferred from R50, R52]</t>
+  </si>
+  <si>
+    <t>(flexibility) Same kWh at lower price and lower CO2 per ton [inferred from R4, R28]</t>
+  </si>
+  <si>
+    <t>(flexibility) Capacity and activation revenue per MW offered [found R1]</t>
+  </si>
+  <si>
+    <t>(procurement and trading) Buys the cheapest tCO2 avoided per year: biomethane premium vs EUA at ~74 €/t [inferred from R36, R10]</t>
+  </si>
+  <si>
+    <t>(investment) Replaces gas steam in low-price power hours and cuts EUA purchases per ton [inferred from R2, R28, R31]</t>
+  </si>
+  <si>
+    <t>(operations) Delivers contracted heat with the least gas per MWh [inferred from R8, R10]</t>
+  </si>
+  <si>
+    <t>(operations) Prices tenant steam at true marginal cost, moves €/ton off Henkel's books [inferred from R3, R15]</t>
+  </si>
+  <si>
+    <t>(operations) Less gas per ton of steam [inferred from R10]</t>
+  </si>
+  <si>
+    <t>R54</t>
+  </si>
+  <si>
+    <t>Whole-plant energy cost 2025, gas and CO2, denominator for criterion (b)</t>
+  </si>
+  <si>
+    <t>EUR per year</t>
+  </si>
+  <si>
+    <t>derived, see reason</t>
+  </si>
+  <si>
+    <t>own calculation from R50, R31, R52, R36</t>
+  </si>
+  <si>
+    <t>right basis for an ETS plant: no BEHG levy, energy tax on CHP fuel largely refunded (my knowledge, not sourced); band check on gross basis: R50 at 56.1 tCO2 per TJ (net) is 1 047 000 MWh net, times 1.11 = 1 162 000 MWh gross = 4.2 million GJ, so the plant sits in band I6 (4 million GJ or over), whose 2025 values are 0.0457 (S1) and 0.0379 (S2); I5 kept as the main row because the site's own gas volume is not public and the yearly averages differ by 8 % (0.0388 vs 0.0418); Eurostat prices are per kWh gross, fuel from R50 is net, convert with 1.11</t>
+  </si>
+  <si>
+    <t>D5 sensitivity year; band I6 values 2024: 0.0332 (S1), 0.0383 (S2)</t>
+  </si>
+  <si>
+    <t>gas: 211 078 tCO2 / 0.2016 tCO2 per MWh (net) = 1 047 000 MWh net × 1.11 = 1 162 000 MWh gross × 0.03875 EUR per kWh (gross, R31) = 45.0 million; CO2: (211 078 − 61 633) × 74 = 11.1 million; total about 56 million</t>
+  </si>
+  <si>
+    <t>fixed before scoring, per D2; whole plant incl. steam and power for third parties, purchased electricity not included (volume unknown); Henkel's own share is 20 to 100 % of it (R15); 5 % = 2.8 million, 1 % = 0.56 million; 0.2016 is the standard 56.1 tCO2 per TJ for natural gas on net calorific value, 1.11 converts net to gross because Eurostat prices are per kWh gross</t>
+  </si>
+  <si>
+    <t>15-min steam and power demand forecast per consumer (Henkel lines, BASF/KLK, district heat) driving CHP unit commitment (incl. district-heat source split, formerly U9)</t>
+  </si>
+  <si>
+    <t>shortlist</t>
+  </si>
+  <si>
+    <t>cut</t>
+  </si>
+  <si>
+    <t>merged into U1</t>
+  </si>
+  <si>
+    <t>ETS compliance forecasting: rolling year-end EUA need and buy-timing per month</t>
+  </si>
+  <si>
+    <t>(procurement and trading) Avoids buying the ~150 kt shortfall at spot in April; spreads purchases over the year to a lower average €/EUA [inferred from R50, R52, R36]</t>
+  </si>
+  <si>
+    <t>R50, R51, R52, R36, R35, R16, R1</t>
+  </si>
+  <si>
+    <t>Monthly verified-emission run-rate, allowance holdings, EUA forward curve, group compliance calendar</t>
+  </si>
+  <si>
+    <t>Group may already forward-buy centrally [guess]; overlaps with #4 if hedging covers EUAs; annual free allocation 61 633 is fixed [found R52], so only timing is optimisable</t>
+  </si>
+  <si>
+    <t>On-site PV and battery: size and dispatch against import price, export value and grid charges</t>
+  </si>
+  <si>
+    <t>(investment) Displaces purchased kWh at ~13 ct and shaves peak charges per ton [inferred from R28, R48]</t>
+  </si>
+  <si>
+    <t>R2, R48, R28, R30, R14, R1</t>
+  </si>
+  <si>
+    <t>Roof and land area, 15-min import profile, grid-connection headroom, CAPEX quotes, export tariff</t>
+  </si>
+  <si>
+    <t>[assumes: roof/land available and grid headroom]; own CHP already covers much of the load [inferred from R48], so PV may mostly displace cheap CHP power, not 13-ct imports; R14 shows 137 122 MWh renewable generation at group level [found], site PV share not known</t>
+  </si>
+  <si>
+    <t>Cut without a score. A cost transfer between Henkel and the tenants, no site saving under D1. Its data (tenant meters, contract formulas) is the first-visit data request.</t>
+  </si>
+  <si>
+    <t>Rests on [assumes: no fixed-price feed-in contract], tier C (a 1). The purchased volume is unknown and peak savings are likely under €0.56 M (b 1). It needs the 15-min import and export data plus the grid contract (c 2). Import and export decisions are the OS's own (d 3). Extension of U2 once the grid contract is known.</t>
+  </si>
+  <si>
+    <t>Rests on [assumes: site procures its own gas and EUAs] (a 1). Hedging lowers the risk and leaves the expected bill unchanged, no net saving under D1 (b 1). It needs volumes and positions from procurement (c 2). A person places the hedges on the OS's analysis (d 2).</t>
+  </si>
+  <si>
+    <t>Rests on [assumes: shiftable electric loads exist] (a 1). Own CHP power dampens the price signal and the products are not power-intensive (b 1). Line load profiles would have to be created (c 1). Shifting loads by the hour is the OS's own decision (d 3).</t>
+  </si>
+  <si>
+    <t>Already started per R10, so reduced to the volume and timing decision. The weakest row is the group target R53 (a 2). A cost of compliance, no net saving under D1 (b 1). It needs biomethane offers and the target path per year (c 2). A person places the purchase (d 2).</t>
+  </si>
+  <si>
+    <t>Rests on [assumes: low-pressure steam share] (a 1). Steam from the CHP costs about €60/MWh in gas and CO2, from an electrode boiler about €130 at 13 ct, it pays only in a few hundred low-price hours (b 1). Capex quotes and steam levels would have to be created (c 1). A one-off investment the OS's data would inform (d 2).</t>
+  </si>
+  <si>
+    <t>The site rows are tier A (a 3). Monitoring alone recovers about 0.5 to 1 % of fuel, €0.3 to 0.56 M with its CO2, at or under the 1 % line (b 1). The control system logs this already (c 3). A person acts on the finding (d 2). Reduced by the already-done rule to the monitoring layer, the efficiency gains themselves are in Henkel's plan (R10).</t>
+  </si>
+  <si>
+    <t>Rests on R35, a tier B price (a 2). Spreading purchases is hedging, it removes risk and leaves the expected cost unchanged, no net saving under D1 (b 1). It needs the emission run-rate plus the registry holdings (c 2). A person places the orders (d 2).</t>
+  </si>
+  <si>
+    <t>Rests on [assumes: roof, land and grid headroom] (a 1). PV displaces the plant's own power, worth about 5.5 ct, and only rarely a 13-ct import, about €0.25 M for 5 MWp (b 1). A roof survey and quotes would have to be created (c 1). A one-off investment the OS's data would inform (d 2).</t>
+  </si>
+  <si>
+    <t>status (shortlist / cut / merged)</t>
+  </si>
+  <si>
+    <t>The site rows are tier A (a 3). A 1 to 3 % fuel saving with its CO2 is €0.56 to 1.7 M a year, my order-of-magnitude guess, checked in calc (b 2). It needs a historian export plus the unit heat rates (c 2). 15-minute unit commitment is what the OS does per R1 (d 3). Takes over the heat dispatch of U9 (D8).</t>
+  </si>
+  <si>
+    <t>Third slot after the tie with U6 at 8 points and (a) 2, U2 has fewer [assumes] tags (D9). The prices are tier B (a 2). 8.6 MW for about 6 000 h at €5 to 15/MWh is €0.26 to 0.8 M, the low end under 1 % (b 1). It needs the unit data plus the gas contract price (c 2). Hourly dispatch of one unit is the OS's own decision (d 3). First step of the market family, U3 and U6 are its extensions.</t>
+  </si>
+  <si>
+    <t>Lost the tie with U2 at 8 points and (a) 2 on the second tie-break, one [assumes] tag on prequalification (D9). The revenue rests on RIZM's own claim R1, external boundary (a 2). About 8 MW at 2025 capacity prices is €0.1 to 0.4 M (b 1). It needs ramp rates and extraction limits from the plant plus aggregator terms (c 2). Offering flexibility by the hour is the OS's own decision (d 3). Extension of U2.</t>
+  </si>
+  <si>
+    <t>Merged into U1 (D8). The heat source split is one of U1's 15-minute unit-commitment decisions, modeled apart it counts the same gas twice. On its own it would have scored 8 with (a) 3. The sale itself is already done, only the hourly split is left. The heat contract data becomes a U1 parameter.</t>
   </si>
 </sst>
 </file>
@@ -1035,9 +1332,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1393,7 +1691,7 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="E1" t="s">
         <v>3</v>
@@ -1404,362 +1702,362 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2" t="s">
         <v>39</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" s="1">
+        <v>46290</v>
+      </c>
+      <c r="F2" t="s">
         <v>40</v>
-      </c>
-      <c r="D2" t="s">
-        <v>41</v>
-      </c>
-      <c r="E2" s="1">
-        <v>46290</v>
-      </c>
-      <c r="F2" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D3" t="s">
+        <v>39</v>
+      </c>
+      <c r="E3" s="1">
+        <v>46290</v>
+      </c>
+      <c r="F3" t="s">
         <v>43</v>
-      </c>
-      <c r="C3" t="s">
-        <v>44</v>
-      </c>
-      <c r="D3" t="s">
-        <v>41</v>
-      </c>
-      <c r="E3" s="1">
-        <v>46290</v>
-      </c>
-      <c r="F3" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D4" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E4" s="1">
         <v>46290</v>
       </c>
       <c r="F4" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B5" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D5" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E5" s="1">
         <v>46290</v>
       </c>
       <c r="F5" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6" s="1">
+        <v>46290</v>
+      </c>
+      <c r="F6" t="s">
         <v>53</v>
-      </c>
-      <c r="C6" t="s">
-        <v>54</v>
-      </c>
-      <c r="D6" t="s">
-        <v>41</v>
-      </c>
-      <c r="E6" s="1">
-        <v>46290</v>
-      </c>
-      <c r="F6" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="B7" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="C7" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D7" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E7" s="1">
         <v>46290</v>
       </c>
       <c r="F7" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="B8" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="C8" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D8" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E8" s="1">
         <v>46290</v>
       </c>
       <c r="F8" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="B9" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="C9" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="D9" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E9" s="1">
         <v>46290</v>
       </c>
       <c r="F9" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="B10" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="C10" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D10" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E10" s="1">
         <v>46290</v>
       </c>
       <c r="F10" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="B11" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="C11" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D11" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E11" s="1">
         <v>46290</v>
       </c>
       <c r="F11" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="B12" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="C12" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="D12" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E12" s="1">
         <v>46290</v>
       </c>
       <c r="F12" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>275</v>
+      </c>
+      <c r="B13" t="s">
+        <v>276</v>
+      </c>
+      <c r="C13" t="s">
+        <v>277</v>
+      </c>
+      <c r="D13" t="s">
         <v>278</v>
       </c>
-      <c r="B13" t="s">
+      <c r="E13" s="1">
+        <v>46290</v>
+      </c>
+      <c r="F13" t="s">
         <v>279</v>
-      </c>
-      <c r="C13" t="s">
-        <v>280</v>
-      </c>
-      <c r="D13" t="s">
-        <v>281</v>
-      </c>
-      <c r="E13" s="1">
-        <v>46290</v>
-      </c>
-      <c r="F13" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="B14" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="C14" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="D14" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E14" s="1">
         <v>46290</v>
       </c>
       <c r="F14" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
+        <v>283</v>
+      </c>
+      <c r="B15" t="s">
+        <v>284</v>
+      </c>
+      <c r="C15" t="s">
+        <v>285</v>
+      </c>
+      <c r="D15" t="s">
+        <v>278</v>
+      </c>
+      <c r="E15" s="1">
+        <v>46290</v>
+      </c>
+      <c r="F15" t="s">
         <v>286</v>
-      </c>
-      <c r="B15" t="s">
-        <v>287</v>
-      </c>
-      <c r="C15" t="s">
-        <v>288</v>
-      </c>
-      <c r="D15" t="s">
-        <v>281</v>
-      </c>
-      <c r="E15" s="1">
-        <v>46290</v>
-      </c>
-      <c r="F15" t="s">
-        <v>289</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="B16" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="C16" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="D16" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E16" s="1">
         <v>46290</v>
       </c>
       <c r="F16" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="B17" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="C17" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="D17" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E17" s="1">
         <v>46290</v>
       </c>
       <c r="F17" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
+        <v>293</v>
+      </c>
+      <c r="B18" t="s">
+        <v>294</v>
+      </c>
+      <c r="C18" t="s">
+        <v>295</v>
+      </c>
+      <c r="D18" t="s">
+        <v>39</v>
+      </c>
+      <c r="E18" s="1">
+        <v>46290</v>
+      </c>
+      <c r="F18" t="s">
         <v>296</v>
-      </c>
-      <c r="B18" t="s">
-        <v>297</v>
-      </c>
-      <c r="C18" t="s">
-        <v>298</v>
-      </c>
-      <c r="D18" t="s">
-        <v>41</v>
-      </c>
-      <c r="E18" s="1">
-        <v>46290</v>
-      </c>
-      <c r="F18" t="s">
-        <v>299</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="B19" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="C19" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="D19" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E19" s="1">
         <v>46290</v>
       </c>
       <c r="F19" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
     </row>
   </sheetData>
@@ -1770,7 +2068,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9BB1BBE5-2A1A-1A4B-BDBA-8116C77369EC}">
-  <dimension ref="A1:O37"/>
+  <dimension ref="A1:O38"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="17.83203125" customWidth="1"/>
@@ -1833,37 +2131,37 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D2" t="s">
         <v>56</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>57</v>
       </c>
-      <c r="D2" t="s">
+      <c r="G2" t="s">
+        <v>41</v>
+      </c>
+      <c r="H2" t="s">
+        <v>42</v>
+      </c>
+      <c r="I2" t="s">
         <v>58</v>
-      </c>
-      <c r="E2" t="s">
-        <v>59</v>
-      </c>
-      <c r="G2" t="s">
-        <v>43</v>
-      </c>
-      <c r="H2" t="s">
-        <v>44</v>
-      </c>
-      <c r="I2" t="s">
-        <v>60</v>
       </c>
       <c r="J2">
         <v>2025</v>
       </c>
       <c r="K2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="L2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M2" s="1">
         <v>46290</v>
@@ -1871,37 +2169,37 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C3" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="G3" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="H3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="I3" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="J3">
         <v>2025</v>
       </c>
       <c r="K3" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="L3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M3" s="1">
         <v>46290</v>
@@ -1909,37 +2207,37 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D4" t="s">
+        <v>56</v>
+      </c>
+      <c r="E4" t="s">
+        <v>57</v>
+      </c>
+      <c r="G4" t="s">
+        <v>41</v>
+      </c>
+      <c r="H4" t="s">
+        <v>42</v>
+      </c>
+      <c r="I4" t="s">
         <v>65</v>
-      </c>
-      <c r="C4" t="s">
-        <v>66</v>
-      </c>
-      <c r="D4" t="s">
-        <v>58</v>
-      </c>
-      <c r="E4" t="s">
-        <v>59</v>
-      </c>
-      <c r="G4" t="s">
-        <v>43</v>
-      </c>
-      <c r="H4" t="s">
-        <v>44</v>
-      </c>
-      <c r="I4" t="s">
-        <v>67</v>
       </c>
       <c r="J4">
         <v>2025</v>
       </c>
       <c r="K4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="L4" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M4" s="1">
         <v>46290</v>
@@ -1947,37 +2245,37 @@
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B5" t="s">
         <v>68</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
+        <v>69</v>
+      </c>
+      <c r="D5" t="s">
+        <v>56</v>
+      </c>
+      <c r="E5" t="s">
+        <v>57</v>
+      </c>
+      <c r="G5" t="s">
+        <v>41</v>
+      </c>
+      <c r="H5" t="s">
+        <v>42</v>
+      </c>
+      <c r="I5" t="s">
         <v>70</v>
-      </c>
-      <c r="C5" t="s">
-        <v>71</v>
-      </c>
-      <c r="D5" t="s">
-        <v>58</v>
-      </c>
-      <c r="E5" t="s">
-        <v>59</v>
-      </c>
-      <c r="G5" t="s">
-        <v>43</v>
-      </c>
-      <c r="H5" t="s">
-        <v>44</v>
-      </c>
-      <c r="I5" t="s">
-        <v>72</v>
       </c>
       <c r="J5">
         <v>2025</v>
       </c>
       <c r="K5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="L5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M5" s="1">
         <v>46290</v>
@@ -1985,37 +2283,37 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B6" t="s">
+        <v>71</v>
+      </c>
+      <c r="C6" t="s">
+        <v>72</v>
+      </c>
+      <c r="D6" t="s">
+        <v>56</v>
+      </c>
+      <c r="E6" t="s">
+        <v>57</v>
+      </c>
+      <c r="G6" t="s">
+        <v>41</v>
+      </c>
+      <c r="H6" t="s">
+        <v>42</v>
+      </c>
+      <c r="I6" t="s">
         <v>73</v>
-      </c>
-      <c r="C6" t="s">
-        <v>74</v>
-      </c>
-      <c r="D6" t="s">
-        <v>58</v>
-      </c>
-      <c r="E6" t="s">
-        <v>59</v>
-      </c>
-      <c r="G6" t="s">
-        <v>43</v>
-      </c>
-      <c r="H6" t="s">
-        <v>44</v>
-      </c>
-      <c r="I6" t="s">
-        <v>75</v>
       </c>
       <c r="J6">
         <v>2025</v>
       </c>
       <c r="K6" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="L6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M6" s="1">
         <v>46290</v>
@@ -2023,78 +2321,78 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>75</v>
+      </c>
+      <c r="B7" t="s">
+        <v>76</v>
+      </c>
+      <c r="C7" t="s">
         <v>77</v>
       </c>
-      <c r="B7" t="s">
+      <c r="D7" t="s">
+        <v>56</v>
+      </c>
+      <c r="E7" t="s">
+        <v>57</v>
+      </c>
+      <c r="G7" t="s">
         <v>78</v>
       </c>
-      <c r="C7" t="s">
+      <c r="H7" t="s">
         <v>79</v>
       </c>
-      <c r="D7" t="s">
-        <v>58</v>
-      </c>
-      <c r="E7" t="s">
-        <v>59</v>
-      </c>
-      <c r="G7" t="s">
+      <c r="I7" t="s">
         <v>80</v>
-      </c>
-      <c r="H7" t="s">
-        <v>81</v>
-      </c>
-      <c r="I7" t="s">
-        <v>82</v>
       </c>
       <c r="J7">
         <v>2026</v>
       </c>
       <c r="K7" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="L7" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M7" s="1">
         <v>46290</v>
       </c>
       <c r="O7" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>83</v>
+      </c>
+      <c r="B8" t="s">
+        <v>84</v>
+      </c>
+      <c r="C8" t="s">
         <v>85</v>
       </c>
-      <c r="B8" t="s">
+      <c r="D8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E8" t="s">
+        <v>57</v>
+      </c>
+      <c r="G8" t="s">
         <v>86</v>
       </c>
-      <c r="C8" t="s">
+      <c r="H8" t="s">
         <v>87</v>
       </c>
-      <c r="D8" t="s">
-        <v>58</v>
-      </c>
-      <c r="E8" t="s">
-        <v>59</v>
-      </c>
-      <c r="G8" t="s">
+      <c r="I8" t="s">
         <v>88</v>
-      </c>
-      <c r="H8" t="s">
-        <v>89</v>
-      </c>
-      <c r="I8" t="s">
-        <v>90</v>
       </c>
       <c r="J8">
         <v>2025</v>
       </c>
       <c r="K8" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="L8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M8" s="1">
         <v>46290</v>
@@ -2102,368 +2400,368 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
+        <v>89</v>
+      </c>
+      <c r="B9" t="s">
+        <v>90</v>
+      </c>
+      <c r="C9" t="s">
         <v>91</v>
       </c>
-      <c r="B9" t="s">
+      <c r="D9" t="s">
+        <v>56</v>
+      </c>
+      <c r="E9" t="s">
+        <v>57</v>
+      </c>
+      <c r="G9" t="s">
+        <v>86</v>
+      </c>
+      <c r="H9" t="s">
+        <v>87</v>
+      </c>
+      <c r="I9" t="s">
         <v>92</v>
-      </c>
-      <c r="C9" t="s">
-        <v>93</v>
-      </c>
-      <c r="D9" t="s">
-        <v>58</v>
-      </c>
-      <c r="E9" t="s">
-        <v>59</v>
-      </c>
-      <c r="G9" t="s">
-        <v>88</v>
-      </c>
-      <c r="H9" t="s">
-        <v>89</v>
-      </c>
-      <c r="I9" t="s">
-        <v>94</v>
       </c>
       <c r="J9">
         <v>2025</v>
       </c>
       <c r="K9" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="L9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M9" s="1">
         <v>46290</v>
       </c>
       <c r="O9" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
+        <v>94</v>
+      </c>
+      <c r="B10" t="s">
+        <v>95</v>
+      </c>
+      <c r="C10" t="s">
         <v>96</v>
       </c>
-      <c r="B10" t="s">
+      <c r="D10" t="s">
+        <v>56</v>
+      </c>
+      <c r="E10" t="s">
         <v>97</v>
       </c>
-      <c r="C10" t="s">
+      <c r="G10" t="s">
+        <v>86</v>
+      </c>
+      <c r="H10" t="s">
+        <v>87</v>
+      </c>
+      <c r="I10" t="s">
         <v>98</v>
-      </c>
-      <c r="D10" t="s">
-        <v>58</v>
-      </c>
-      <c r="E10" t="s">
-        <v>99</v>
-      </c>
-      <c r="G10" t="s">
-        <v>88</v>
-      </c>
-      <c r="H10" t="s">
-        <v>89</v>
-      </c>
-      <c r="I10" t="s">
-        <v>100</v>
       </c>
       <c r="J10">
         <v>2025</v>
       </c>
       <c r="K10" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="L10" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M10" s="1">
         <v>46290</v>
       </c>
       <c r="O10" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
+        <v>101</v>
+      </c>
+      <c r="B11" t="s">
+        <v>102</v>
+      </c>
+      <c r="C11" t="s">
         <v>103</v>
       </c>
-      <c r="B11" t="s">
+      <c r="D11" t="s">
+        <v>56</v>
+      </c>
+      <c r="E11" t="s">
+        <v>97</v>
+      </c>
+      <c r="G11" t="s">
         <v>104</v>
       </c>
-      <c r="C11" t="s">
+      <c r="H11" t="s">
+        <v>87</v>
+      </c>
+      <c r="I11" t="s">
         <v>105</v>
-      </c>
-      <c r="D11" t="s">
-        <v>58</v>
-      </c>
-      <c r="E11" t="s">
-        <v>99</v>
-      </c>
-      <c r="G11" t="s">
-        <v>106</v>
-      </c>
-      <c r="H11" t="s">
-        <v>89</v>
-      </c>
-      <c r="I11" t="s">
-        <v>107</v>
       </c>
       <c r="J11">
         <v>2025</v>
       </c>
       <c r="K11" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="L11" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M11" s="1">
         <v>46290</v>
       </c>
       <c r="O11" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
+        <v>108</v>
+      </c>
+      <c r="B12" t="s">
+        <v>109</v>
+      </c>
+      <c r="C12" t="s">
         <v>110</v>
       </c>
-      <c r="B12" t="s">
+      <c r="D12" t="s">
+        <v>56</v>
+      </c>
+      <c r="E12" t="s">
         <v>111</v>
       </c>
-      <c r="C12" t="s">
+      <c r="G12" t="s">
         <v>112</v>
       </c>
-      <c r="D12" t="s">
-        <v>58</v>
-      </c>
-      <c r="E12" t="s">
+      <c r="H12" t="s">
+        <v>87</v>
+      </c>
+      <c r="I12" t="s">
         <v>113</v>
-      </c>
-      <c r="G12" t="s">
-        <v>114</v>
-      </c>
-      <c r="H12" t="s">
-        <v>89</v>
-      </c>
-      <c r="I12" t="s">
-        <v>115</v>
       </c>
       <c r="J12">
         <v>2025</v>
       </c>
       <c r="K12" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="L12" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M12" s="1">
         <v>46290</v>
       </c>
       <c r="O12" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>115</v>
+      </c>
+      <c r="B13" t="s">
+        <v>116</v>
+      </c>
+      <c r="C13" t="s">
         <v>117</v>
       </c>
-      <c r="B13" t="s">
+      <c r="D13" t="s">
+        <v>56</v>
+      </c>
+      <c r="E13" t="s">
         <v>118</v>
       </c>
-      <c r="C13" t="s">
+      <c r="G13" t="s">
+        <v>112</v>
+      </c>
+      <c r="H13" t="s">
+        <v>87</v>
+      </c>
+      <c r="I13" t="s">
         <v>119</v>
-      </c>
-      <c r="D13" t="s">
-        <v>58</v>
-      </c>
-      <c r="E13" t="s">
-        <v>120</v>
-      </c>
-      <c r="G13" t="s">
-        <v>114</v>
-      </c>
-      <c r="H13" t="s">
-        <v>89</v>
-      </c>
-      <c r="I13" t="s">
-        <v>121</v>
       </c>
       <c r="J13">
         <v>2025</v>
       </c>
       <c r="K13" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="L13" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M13" s="1">
         <v>46290</v>
       </c>
       <c r="O13" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
+        <v>121</v>
+      </c>
+      <c r="B14" t="s">
+        <v>122</v>
+      </c>
+      <c r="C14" t="s">
         <v>123</v>
       </c>
-      <c r="B14" t="s">
+      <c r="D14" t="s">
+        <v>56</v>
+      </c>
+      <c r="E14" t="s">
+        <v>111</v>
+      </c>
+      <c r="G14" t="s">
+        <v>112</v>
+      </c>
+      <c r="H14" t="s">
+        <v>87</v>
+      </c>
+      <c r="I14" t="s">
         <v>124</v>
-      </c>
-      <c r="C14" t="s">
-        <v>125</v>
-      </c>
-      <c r="D14" t="s">
-        <v>58</v>
-      </c>
-      <c r="E14" t="s">
-        <v>113</v>
-      </c>
-      <c r="G14" t="s">
-        <v>114</v>
-      </c>
-      <c r="H14" t="s">
-        <v>89</v>
-      </c>
-      <c r="I14" t="s">
-        <v>126</v>
       </c>
       <c r="J14">
         <v>2025</v>
       </c>
       <c r="K14" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="L14" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M14" s="1">
         <v>46290</v>
       </c>
       <c r="O14" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
+        <v>126</v>
+      </c>
+      <c r="B15" t="s">
+        <v>127</v>
+      </c>
+      <c r="C15" t="s">
         <v>128</v>
       </c>
-      <c r="B15" t="s">
+      <c r="D15" t="s">
+        <v>56</v>
+      </c>
+      <c r="E15" t="s">
         <v>129</v>
       </c>
-      <c r="C15" t="s">
+      <c r="G15" t="s">
         <v>130</v>
       </c>
-      <c r="D15" t="s">
-        <v>58</v>
-      </c>
-      <c r="E15" t="s">
+      <c r="H15" t="s">
+        <v>87</v>
+      </c>
+      <c r="I15" t="s">
         <v>131</v>
-      </c>
-      <c r="G15" t="s">
-        <v>132</v>
-      </c>
-      <c r="H15" t="s">
-        <v>89</v>
-      </c>
-      <c r="I15" t="s">
-        <v>133</v>
       </c>
       <c r="J15">
         <v>2025</v>
       </c>
       <c r="K15" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="L15" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M15" s="1">
         <v>46290</v>
       </c>
       <c r="O15" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
+        <v>133</v>
+      </c>
+      <c r="B16" t="s">
+        <v>134</v>
+      </c>
+      <c r="C16" t="s">
         <v>135</v>
       </c>
-      <c r="B16" t="s">
+      <c r="D16" t="s">
         <v>136</v>
       </c>
-      <c r="C16" t="s">
+      <c r="E16" t="s">
         <v>137</v>
       </c>
-      <c r="D16" t="s">
+      <c r="F16" t="s">
         <v>138</v>
       </c>
-      <c r="E16" t="s">
+      <c r="G16" t="s">
         <v>139</v>
       </c>
-      <c r="F16" t="s">
+      <c r="H16" t="s">
         <v>140</v>
       </c>
-      <c r="G16" t="s">
-        <v>141</v>
-      </c>
-      <c r="H16" t="s">
-        <v>142</v>
-      </c>
       <c r="I16" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="J16">
         <v>2025</v>
       </c>
       <c r="K16" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="L16" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="M16" s="1">
         <v>46290</v>
       </c>
       <c r="O16" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
+        <v>143</v>
+      </c>
+      <c r="B17" t="s">
+        <v>144</v>
+      </c>
+      <c r="C17" t="s">
         <v>145</v>
       </c>
-      <c r="B17" t="s">
+      <c r="D17" t="s">
+        <v>56</v>
+      </c>
+      <c r="E17" t="s">
+        <v>57</v>
+      </c>
+      <c r="G17" t="s">
         <v>146</v>
       </c>
-      <c r="C17" t="s">
-        <v>147</v>
-      </c>
-      <c r="D17" t="s">
-        <v>58</v>
-      </c>
-      <c r="E17" t="s">
-        <v>59</v>
-      </c>
-      <c r="G17" t="s">
-        <v>148</v>
-      </c>
       <c r="H17" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="I17" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="J17">
         <v>2025</v>
       </c>
       <c r="K17" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="L17" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M17" s="1">
         <v>46290</v>
@@ -2471,669 +2769,669 @@
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
+        <v>147</v>
+      </c>
+      <c r="B18" t="s">
+        <v>148</v>
+      </c>
+      <c r="C18" t="s">
         <v>149</v>
       </c>
-      <c r="B18" t="s">
+      <c r="D18" t="s">
+        <v>56</v>
+      </c>
+      <c r="E18" t="s">
+        <v>57</v>
+      </c>
+      <c r="G18" t="s">
+        <v>104</v>
+      </c>
+      <c r="H18" t="s">
+        <v>87</v>
+      </c>
+      <c r="I18" t="s">
         <v>150</v>
-      </c>
-      <c r="C18" t="s">
-        <v>151</v>
-      </c>
-      <c r="D18" t="s">
-        <v>58</v>
-      </c>
-      <c r="E18" t="s">
-        <v>59</v>
-      </c>
-      <c r="G18" t="s">
-        <v>106</v>
-      </c>
-      <c r="H18" t="s">
-        <v>89</v>
-      </c>
-      <c r="I18" t="s">
-        <v>152</v>
       </c>
       <c r="J18">
         <v>2025</v>
       </c>
       <c r="K18" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="L18" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M18" s="1">
         <v>46290</v>
       </c>
       <c r="O18" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
+        <v>152</v>
+      </c>
+      <c r="B19" t="s">
+        <v>153</v>
+      </c>
+      <c r="C19" t="s">
         <v>154</v>
       </c>
-      <c r="B19" t="s">
+      <c r="D19" t="s">
+        <v>56</v>
+      </c>
+      <c r="E19" t="s">
         <v>155</v>
       </c>
-      <c r="C19" t="s">
+      <c r="G19" t="s">
         <v>156</v>
       </c>
-      <c r="D19" t="s">
-        <v>58</v>
-      </c>
-      <c r="E19" t="s">
+      <c r="H19" t="s">
         <v>157</v>
       </c>
-      <c r="G19" t="s">
+      <c r="I19" t="s">
         <v>158</v>
-      </c>
-      <c r="H19" t="s">
-        <v>159</v>
-      </c>
-      <c r="I19" t="s">
-        <v>160</v>
       </c>
       <c r="J19">
         <v>2025</v>
       </c>
       <c r="K19" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="L19" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="M19" s="1">
         <v>46290</v>
       </c>
       <c r="O19" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
+        <v>160</v>
+      </c>
+      <c r="B20" t="s">
+        <v>161</v>
+      </c>
+      <c r="C20" t="s">
         <v>162</v>
       </c>
-      <c r="B20" t="s">
+      <c r="D20" t="s">
+        <v>56</v>
+      </c>
+      <c r="E20" t="s">
+        <v>155</v>
+      </c>
+      <c r="G20" t="s">
+        <v>156</v>
+      </c>
+      <c r="H20" t="s">
+        <v>157</v>
+      </c>
+      <c r="I20" t="s">
         <v>163</v>
-      </c>
-      <c r="C20" t="s">
-        <v>164</v>
-      </c>
-      <c r="D20" t="s">
-        <v>58</v>
-      </c>
-      <c r="E20" t="s">
-        <v>157</v>
-      </c>
-      <c r="G20" t="s">
-        <v>158</v>
-      </c>
-      <c r="H20" t="s">
-        <v>159</v>
-      </c>
-      <c r="I20" t="s">
-        <v>165</v>
       </c>
       <c r="J20">
         <v>2024</v>
       </c>
       <c r="K20" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="L20" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="M20" s="1">
         <v>46290</v>
       </c>
       <c r="O20" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
+        <v>165</v>
+      </c>
+      <c r="B21" t="s">
+        <v>166</v>
+      </c>
+      <c r="C21" t="s">
         <v>167</v>
       </c>
-      <c r="B21" t="s">
+      <c r="D21" t="s">
+        <v>56</v>
+      </c>
+      <c r="E21" t="s">
+        <v>155</v>
+      </c>
+      <c r="G21" t="s">
+        <v>156</v>
+      </c>
+      <c r="H21" t="s">
+        <v>157</v>
+      </c>
+      <c r="I21" t="s">
         <v>168</v>
-      </c>
-      <c r="C21" t="s">
-        <v>169</v>
-      </c>
-      <c r="D21" t="s">
-        <v>58</v>
-      </c>
-      <c r="E21" t="s">
-        <v>157</v>
-      </c>
-      <c r="G21" t="s">
-        <v>158</v>
-      </c>
-      <c r="H21" t="s">
-        <v>159</v>
-      </c>
-      <c r="I21" t="s">
-        <v>170</v>
       </c>
       <c r="J21">
         <v>2025</v>
       </c>
       <c r="K21" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="L21" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="M21" s="1">
         <v>46290</v>
       </c>
       <c r="O21" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
+        <v>170</v>
+      </c>
+      <c r="B22" t="s">
+        <v>171</v>
+      </c>
+      <c r="C22" t="s">
         <v>172</v>
       </c>
-      <c r="B22" t="s">
+      <c r="D22" t="s">
+        <v>56</v>
+      </c>
+      <c r="E22" t="s">
         <v>173</v>
       </c>
-      <c r="C22" t="s">
+      <c r="G22" t="s">
         <v>174</v>
       </c>
-      <c r="D22" t="s">
-        <v>58</v>
-      </c>
-      <c r="E22" t="s">
+      <c r="H22" t="s">
         <v>175</v>
       </c>
-      <c r="G22" t="s">
+      <c r="I22" t="s">
         <v>176</v>
-      </c>
-      <c r="H22" t="s">
-        <v>177</v>
-      </c>
-      <c r="I22" t="s">
-        <v>178</v>
       </c>
       <c r="J22">
         <v>2025</v>
       </c>
       <c r="K22" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="L22" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="M22" s="1">
         <v>46290</v>
       </c>
       <c r="O22" t="s">
-        <v>179</v>
+        <v>384</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
+        <v>177</v>
+      </c>
+      <c r="B23" t="s">
+        <v>178</v>
+      </c>
+      <c r="C23" t="s">
+        <v>179</v>
+      </c>
+      <c r="D23" t="s">
+        <v>56</v>
+      </c>
+      <c r="E23" t="s">
+        <v>173</v>
+      </c>
+      <c r="G23" t="s">
+        <v>174</v>
+      </c>
+      <c r="H23" t="s">
+        <v>175</v>
+      </c>
+      <c r="I23" t="s">
         <v>180</v>
-      </c>
-      <c r="B23" t="s">
-        <v>181</v>
-      </c>
-      <c r="C23" t="s">
-        <v>182</v>
-      </c>
-      <c r="D23" t="s">
-        <v>58</v>
-      </c>
-      <c r="E23" t="s">
-        <v>175</v>
-      </c>
-      <c r="G23" t="s">
-        <v>176</v>
-      </c>
-      <c r="H23" t="s">
-        <v>177</v>
-      </c>
-      <c r="I23" t="s">
-        <v>183</v>
       </c>
       <c r="J23">
         <v>2024</v>
       </c>
       <c r="K23" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="L23" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="M23" s="1">
         <v>46290</v>
       </c>
       <c r="O23" t="s">
-        <v>166</v>
+        <v>385</v>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="B24" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="C24">
         <v>65</v>
       </c>
       <c r="D24" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E24" t="s">
+        <v>183</v>
+      </c>
+      <c r="G24" t="s">
+        <v>184</v>
+      </c>
+      <c r="H24" t="s">
+        <v>185</v>
+      </c>
+      <c r="I24" t="s">
         <v>186</v>
-      </c>
-      <c r="G24" t="s">
-        <v>187</v>
-      </c>
-      <c r="H24" t="s">
-        <v>188</v>
-      </c>
-      <c r="I24" t="s">
-        <v>189</v>
       </c>
       <c r="J24">
         <v>2024</v>
       </c>
       <c r="K24" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="L24" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="M24" s="1">
         <v>46290</v>
       </c>
       <c r="O24" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="B25" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="C25" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="D25">
         <v>74</v>
       </c>
       <c r="E25" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="F25" t="s">
+        <v>191</v>
+      </c>
+      <c r="G25" t="s">
+        <v>192</v>
+      </c>
+      <c r="H25" t="s">
+        <v>193</v>
+      </c>
+      <c r="I25" t="s">
         <v>194</v>
-      </c>
-      <c r="G25" t="s">
-        <v>195</v>
-      </c>
-      <c r="H25" t="s">
-        <v>196</v>
-      </c>
-      <c r="I25" t="s">
-        <v>197</v>
       </c>
       <c r="J25">
         <v>2025</v>
       </c>
       <c r="K25" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="L25" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M25" s="1">
         <v>46290</v>
       </c>
       <c r="O25" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="B26" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="C26">
         <v>89</v>
       </c>
       <c r="D26" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E26" t="s">
+        <v>198</v>
+      </c>
+      <c r="G26" t="s">
+        <v>199</v>
+      </c>
+      <c r="H26" t="s">
+        <v>200</v>
+      </c>
+      <c r="I26" t="s">
         <v>201</v>
-      </c>
-      <c r="G26" t="s">
-        <v>202</v>
-      </c>
-      <c r="H26" t="s">
-        <v>203</v>
-      </c>
-      <c r="I26" t="s">
-        <v>204</v>
       </c>
       <c r="J26">
         <v>2023</v>
       </c>
       <c r="K26" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="L26" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="M26" s="1">
         <v>46290</v>
       </c>
       <c r="O26" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="B27" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="C27">
         <v>85</v>
       </c>
       <c r="D27" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E27" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="G27" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H27" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="I27" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="J27">
         <v>2023</v>
       </c>
       <c r="K27" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="L27" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="M27" s="1">
         <v>46290</v>
       </c>
       <c r="O27" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
+        <v>208</v>
+      </c>
+      <c r="B28" t="s">
+        <v>209</v>
+      </c>
+      <c r="C28" t="s">
+        <v>210</v>
+      </c>
+      <c r="D28" t="s">
+        <v>56</v>
+      </c>
+      <c r="E28" t="s">
+        <v>57</v>
+      </c>
+      <c r="G28" t="s">
         <v>211</v>
       </c>
-      <c r="B28" t="s">
+      <c r="H28" t="s">
         <v>212</v>
       </c>
-      <c r="C28" t="s">
+      <c r="I28" t="s">
         <v>213</v>
-      </c>
-      <c r="D28" t="s">
-        <v>58</v>
-      </c>
-      <c r="E28" t="s">
-        <v>59</v>
-      </c>
-      <c r="G28" t="s">
-        <v>214</v>
-      </c>
-      <c r="H28" t="s">
-        <v>215</v>
-      </c>
-      <c r="I28" t="s">
-        <v>216</v>
       </c>
       <c r="J28">
         <v>2014</v>
       </c>
       <c r="K28" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="L28" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="M28" s="1">
         <v>46290</v>
       </c>
       <c r="O28" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
+        <v>215</v>
+      </c>
+      <c r="B29" t="s">
+        <v>216</v>
+      </c>
+      <c r="C29" t="s">
+        <v>302</v>
+      </c>
+      <c r="D29" t="s">
+        <v>56</v>
+      </c>
+      <c r="E29" t="s">
+        <v>217</v>
+      </c>
+      <c r="G29" t="s">
         <v>218</v>
       </c>
-      <c r="B29" t="s">
+      <c r="H29" t="s">
         <v>219</v>
       </c>
-      <c r="C29" t="s">
-        <v>305</v>
-      </c>
-      <c r="D29" t="s">
-        <v>58</v>
-      </c>
-      <c r="E29" t="s">
+      <c r="I29" t="s">
         <v>220</v>
-      </c>
-      <c r="G29" t="s">
-        <v>221</v>
-      </c>
-      <c r="H29" t="s">
-        <v>222</v>
-      </c>
-      <c r="I29" t="s">
-        <v>223</v>
       </c>
       <c r="J29">
         <v>2026</v>
       </c>
       <c r="K29" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="L29" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M29" s="1">
         <v>46290</v>
       </c>
       <c r="O29" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
+        <v>222</v>
+      </c>
+      <c r="B30" t="s">
+        <v>223</v>
+      </c>
+      <c r="C30" t="s">
+        <v>303</v>
+      </c>
+      <c r="D30" t="s">
+        <v>56</v>
+      </c>
+      <c r="E30" t="s">
+        <v>217</v>
+      </c>
+      <c r="G30" t="s">
+        <v>224</v>
+      </c>
+      <c r="H30" t="s">
+        <v>219</v>
+      </c>
+      <c r="I30" t="s">
         <v>225</v>
-      </c>
-      <c r="B30" t="s">
-        <v>226</v>
-      </c>
-      <c r="C30" t="s">
-        <v>306</v>
-      </c>
-      <c r="D30" t="s">
-        <v>58</v>
-      </c>
-      <c r="E30" t="s">
-        <v>220</v>
-      </c>
-      <c r="G30" t="s">
-        <v>227</v>
-      </c>
-      <c r="H30" t="s">
-        <v>222</v>
-      </c>
-      <c r="I30" t="s">
-        <v>228</v>
       </c>
       <c r="J30">
         <v>2026</v>
       </c>
       <c r="K30" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="L30" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M30" s="1">
         <v>46290</v>
       </c>
       <c r="O30" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="B31" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="C31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="D31" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E31" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="G31" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="H31" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="I31" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="J31">
         <v>2025</v>
       </c>
       <c r="K31" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="L31" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M31" s="1">
         <v>46290</v>
       </c>
       <c r="O31" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
+        <v>231</v>
+      </c>
+      <c r="B32" t="s">
+        <v>232</v>
+      </c>
+      <c r="C32" t="s">
+        <v>305</v>
+      </c>
+      <c r="D32" t="s">
+        <v>56</v>
+      </c>
+      <c r="E32" t="s">
+        <v>217</v>
+      </c>
+      <c r="G32" t="s">
+        <v>233</v>
+      </c>
+      <c r="H32" t="s">
+        <v>219</v>
+      </c>
+      <c r="I32" t="s">
         <v>234</v>
-      </c>
-      <c r="B32" t="s">
-        <v>235</v>
-      </c>
-      <c r="C32" t="s">
-        <v>308</v>
-      </c>
-      <c r="D32" t="s">
-        <v>58</v>
-      </c>
-      <c r="E32" t="s">
-        <v>220</v>
-      </c>
-      <c r="G32" t="s">
-        <v>236</v>
-      </c>
-      <c r="H32" t="s">
-        <v>222</v>
-      </c>
-      <c r="I32" t="s">
-        <v>237</v>
       </c>
       <c r="J32">
         <v>2026</v>
       </c>
       <c r="K32" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="L32" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M32" s="1">
         <v>46290</v>
       </c>
       <c r="O32" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
+        <v>236</v>
+      </c>
+      <c r="B33" t="s">
+        <v>237</v>
+      </c>
+      <c r="C33" t="s">
+        <v>238</v>
+      </c>
+      <c r="D33" t="s">
+        <v>56</v>
+      </c>
+      <c r="E33" t="s">
+        <v>57</v>
+      </c>
+      <c r="G33" t="s">
         <v>239</v>
       </c>
-      <c r="B33" t="s">
+      <c r="H33" t="s">
         <v>240</v>
       </c>
-      <c r="C33" t="s">
+      <c r="I33" t="s">
         <v>241</v>
-      </c>
-      <c r="D33" t="s">
-        <v>58</v>
-      </c>
-      <c r="E33" t="s">
-        <v>59</v>
-      </c>
-      <c r="G33" t="s">
-        <v>242</v>
-      </c>
-      <c r="H33" t="s">
-        <v>243</v>
-      </c>
-      <c r="I33" t="s">
-        <v>244</v>
       </c>
       <c r="J33">
         <v>2025</v>
       </c>
       <c r="K33" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="L33" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M33" s="1">
         <v>46290</v>
       </c>
       <c r="O33" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="B34" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="C34">
         <v>211.078</v>
@@ -3142,39 +3440,39 @@
         <v>211078</v>
       </c>
       <c r="E34" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="G34" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="H34" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="I34" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="J34">
         <v>2025</v>
       </c>
       <c r="K34" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="L34" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M34" s="1">
         <v>46290</v>
       </c>
       <c r="O34" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="B35" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="C35">
         <v>229.042</v>
@@ -3183,39 +3481,39 @@
         <v>229042</v>
       </c>
       <c r="E35" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="G35" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="H35" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="I35" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="J35">
         <v>2024</v>
       </c>
       <c r="K35" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="L35" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M35" s="1">
         <v>46290</v>
       </c>
       <c r="O35" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="B36" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="C36">
         <v>61.633000000000003</v>
@@ -3224,72 +3522,116 @@
         <v>61633</v>
       </c>
       <c r="E36" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="G36" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="H36" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="I36" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="J36">
         <v>2025</v>
       </c>
       <c r="K36" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="L36" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M36" s="1">
         <v>46290</v>
       </c>
       <c r="O36" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="B37" t="s">
+        <v>309</v>
+      </c>
+      <c r="C37" t="s">
+        <v>310</v>
+      </c>
+      <c r="D37" t="s">
+        <v>56</v>
+      </c>
+      <c r="E37" t="s">
+        <v>111</v>
+      </c>
+      <c r="G37" t="s">
+        <v>311</v>
+      </c>
+      <c r="H37" t="s">
+        <v>87</v>
+      </c>
+      <c r="I37" t="s">
         <v>312</v>
-      </c>
-      <c r="C37" t="s">
-        <v>313</v>
-      </c>
-      <c r="D37" t="s">
-        <v>58</v>
-      </c>
-      <c r="E37" t="s">
-        <v>113</v>
-      </c>
-      <c r="G37" t="s">
-        <v>314</v>
-      </c>
-      <c r="H37" t="s">
-        <v>89</v>
-      </c>
-      <c r="I37" t="s">
-        <v>315</v>
       </c>
       <c r="J37">
         <v>2025</v>
       </c>
       <c r="K37" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="L37" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M37" s="1">
         <v>46290</v>
       </c>
       <c r="O37" t="s">
-        <v>316</v>
+        <v>313</v>
+      </c>
+    </row>
+    <row r="38" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>379</v>
+      </c>
+      <c r="B38" t="s">
+        <v>380</v>
+      </c>
+      <c r="C38" t="s">
+        <v>386</v>
+      </c>
+      <c r="D38">
+        <v>56000000</v>
+      </c>
+      <c r="E38" t="s">
+        <v>381</v>
+      </c>
+      <c r="F38" t="s">
+        <v>382</v>
+      </c>
+      <c r="G38" t="s">
+        <v>383</v>
+      </c>
+      <c r="H38" t="s">
+        <v>140</v>
+      </c>
+      <c r="I38" t="s">
+        <v>140</v>
+      </c>
+      <c r="J38">
+        <v>2025</v>
+      </c>
+      <c r="K38" t="s">
+        <v>81</v>
+      </c>
+      <c r="L38" t="s">
+        <v>141</v>
+      </c>
+      <c r="M38" s="1">
+        <v>46291</v>
+      </c>
+      <c r="O38" t="s">
+        <v>387</v>
       </c>
     </row>
   </sheetData>
@@ -3300,8 +3642,15 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{016B0643-83A2-AA4F-8C67-1D83CAF37A07}">
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="19.6640625" customWidth="1"/>
+    <col min="3" max="3" width="19.5" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="14.1640625" customWidth="1"/>
+    <col min="6" max="6" width="20.1640625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -3334,33 +3683,621 @@
       <c r="J1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="2" t="s">
         <v>26</v>
       </c>
       <c r="L1" t="s">
         <v>27</v>
       </c>
       <c r="M1" t="s">
-        <v>28</v>
+        <v>411</v>
       </c>
       <c r="N1" t="s">
-        <v>29</v>
+        <v>314</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>36</v>
+        <v>34</v>
+      </c>
+      <c r="B2" t="s">
+        <v>388</v>
+      </c>
+      <c r="C2" t="s">
+        <v>368</v>
+      </c>
+      <c r="D2" t="s">
+        <v>315</v>
+      </c>
+      <c r="E2" t="s">
+        <v>316</v>
+      </c>
+      <c r="F2" t="s">
+        <v>317</v>
+      </c>
+      <c r="G2">
+        <v>3</v>
+      </c>
+      <c r="H2" s="2">
+        <v>2</v>
+      </c>
+      <c r="I2">
+        <v>2</v>
+      </c>
+      <c r="J2">
+        <v>3</v>
+      </c>
+      <c r="K2" s="2">
+        <f>SUM($G2:$J2)</f>
+        <v>10</v>
+      </c>
+      <c r="L2">
+        <v>1</v>
+      </c>
+      <c r="M2" t="s">
+        <v>389</v>
+      </c>
+      <c r="N2" t="s">
+        <v>412</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>37</v>
+        <v>35</v>
+      </c>
+      <c r="B3" t="s">
+        <v>318</v>
+      </c>
+      <c r="C3" t="s">
+        <v>369</v>
+      </c>
+      <c r="D3" t="s">
+        <v>319</v>
+      </c>
+      <c r="E3" t="s">
+        <v>320</v>
+      </c>
+      <c r="F3" t="s">
+        <v>321</v>
+      </c>
+      <c r="G3">
+        <v>2</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>2</v>
+      </c>
+      <c r="J3">
+        <v>3</v>
+      </c>
+      <c r="K3" s="2">
+        <f t="shared" ref="K3:K14" si="0">SUM($G3:$J3)</f>
+        <v>8</v>
+      </c>
+      <c r="L3">
+        <v>3</v>
+      </c>
+      <c r="M3" t="s">
+        <v>389</v>
+      </c>
+      <c r="N3" t="s">
+        <v>413</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>38</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="B4" t="s">
+        <v>322</v>
+      </c>
+      <c r="C4" t="s">
+        <v>370</v>
+      </c>
+      <c r="D4" t="s">
+        <v>323</v>
+      </c>
+      <c r="E4" t="s">
+        <v>324</v>
+      </c>
+      <c r="F4" t="s">
+        <v>325</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4">
+        <v>2</v>
+      </c>
+      <c r="J4">
+        <v>3</v>
+      </c>
+      <c r="K4" s="2">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="L4">
+        <v>7</v>
+      </c>
+      <c r="M4" t="s">
+        <v>390</v>
+      </c>
+      <c r="N4" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>326</v>
+      </c>
+      <c r="B5" t="s">
+        <v>327</v>
+      </c>
+      <c r="C5" t="s">
+        <v>371</v>
+      </c>
+      <c r="D5" t="s">
+        <v>328</v>
+      </c>
+      <c r="E5" t="s">
+        <v>329</v>
+      </c>
+      <c r="F5" t="s">
+        <v>330</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5">
+        <v>2</v>
+      </c>
+      <c r="J5">
+        <v>2</v>
+      </c>
+      <c r="K5" s="2">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="L5">
+        <v>8</v>
+      </c>
+      <c r="M5" t="s">
+        <v>390</v>
+      </c>
+      <c r="N5" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>331</v>
+      </c>
+      <c r="B6" t="s">
+        <v>332</v>
+      </c>
+      <c r="C6" t="s">
+        <v>372</v>
+      </c>
+      <c r="D6" t="s">
+        <v>333</v>
+      </c>
+      <c r="E6" t="s">
+        <v>334</v>
+      </c>
+      <c r="F6" t="s">
+        <v>335</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6">
+        <v>1</v>
+      </c>
+      <c r="J6">
+        <v>3</v>
+      </c>
+      <c r="K6" s="2">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="L6">
+        <v>8</v>
+      </c>
+      <c r="M6" t="s">
+        <v>390</v>
+      </c>
+      <c r="N6" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>336</v>
+      </c>
+      <c r="B7" t="s">
+        <v>337</v>
+      </c>
+      <c r="C7" t="s">
+        <v>373</v>
+      </c>
+      <c r="D7" t="s">
+        <v>338</v>
+      </c>
+      <c r="E7" t="s">
+        <v>339</v>
+      </c>
+      <c r="F7" t="s">
+        <v>340</v>
+      </c>
+      <c r="G7">
+        <v>2</v>
+      </c>
+      <c r="H7">
+        <v>1</v>
+      </c>
+      <c r="I7">
+        <v>2</v>
+      </c>
+      <c r="J7">
+        <v>3</v>
+      </c>
+      <c r="K7" s="2">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="L7">
+        <v>4</v>
+      </c>
+      <c r="M7" t="s">
+        <v>390</v>
+      </c>
+      <c r="N7" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>341</v>
+      </c>
+      <c r="B8" t="s">
+        <v>342</v>
+      </c>
+      <c r="C8" t="s">
+        <v>374</v>
+      </c>
+      <c r="D8" t="s">
+        <v>343</v>
+      </c>
+      <c r="E8" t="s">
+        <v>344</v>
+      </c>
+      <c r="F8" t="s">
+        <v>345</v>
+      </c>
+      <c r="G8">
+        <v>2</v>
+      </c>
+      <c r="H8">
+        <v>1</v>
+      </c>
+      <c r="I8">
+        <v>2</v>
+      </c>
+      <c r="J8">
+        <v>2</v>
+      </c>
+      <c r="K8" s="2">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="L8">
+        <v>5</v>
+      </c>
+      <c r="M8" t="s">
+        <v>390</v>
+      </c>
+      <c r="N8" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>346</v>
+      </c>
+      <c r="B9" t="s">
+        <v>347</v>
+      </c>
+      <c r="C9" t="s">
+        <v>375</v>
+      </c>
+      <c r="D9" t="s">
+        <v>348</v>
+      </c>
+      <c r="E9" t="s">
+        <v>349</v>
+      </c>
+      <c r="F9" t="s">
+        <v>350</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9">
+        <v>1</v>
+      </c>
+      <c r="I9">
+        <v>1</v>
+      </c>
+      <c r="J9">
+        <v>2</v>
+      </c>
+      <c r="K9" s="2">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="L9">
+        <v>10</v>
+      </c>
+      <c r="M9" t="s">
+        <v>390</v>
+      </c>
+      <c r="N9" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>351</v>
+      </c>
+      <c r="B10" t="s">
+        <v>352</v>
+      </c>
+      <c r="C10" t="s">
+        <v>376</v>
+      </c>
+      <c r="D10" t="s">
+        <v>353</v>
+      </c>
+      <c r="E10" t="s">
+        <v>354</v>
+      </c>
+      <c r="F10" t="s">
+        <v>355</v>
+      </c>
+      <c r="G10">
+        <v>3</v>
+      </c>
+      <c r="H10">
+        <v>1</v>
+      </c>
+      <c r="I10">
+        <v>2</v>
+      </c>
+      <c r="J10">
+        <v>2</v>
+      </c>
+      <c r="K10" s="2">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="M10" t="s">
+        <v>391</v>
+      </c>
+      <c r="N10" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>356</v>
+      </c>
+      <c r="B11" t="s">
+        <v>357</v>
+      </c>
+      <c r="C11" t="s">
+        <v>377</v>
+      </c>
+      <c r="D11" t="s">
+        <v>358</v>
+      </c>
+      <c r="E11" t="s">
+        <v>359</v>
+      </c>
+      <c r="F11" t="s">
+        <v>360</v>
+      </c>
+      <c r="K11" s="2"/>
+      <c r="M11" t="s">
+        <v>390</v>
+      </c>
+      <c r="N11" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>361</v>
+      </c>
+      <c r="B12" t="s">
+        <v>362</v>
+      </c>
+      <c r="C12" t="s">
+        <v>378</v>
+      </c>
+      <c r="D12" t="s">
+        <v>363</v>
+      </c>
+      <c r="E12" t="s">
+        <v>364</v>
+      </c>
+      <c r="F12" t="s">
+        <v>365</v>
+      </c>
+      <c r="G12">
+        <v>3</v>
+      </c>
+      <c r="H12">
+        <v>1</v>
+      </c>
+      <c r="I12">
+        <v>3</v>
+      </c>
+      <c r="J12">
+        <v>2</v>
+      </c>
+      <c r="K12" s="2">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+      <c r="L12">
+        <v>2</v>
+      </c>
+      <c r="M12" t="s">
+        <v>389</v>
+      </c>
+      <c r="N12" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>366</v>
+      </c>
+      <c r="B13" t="s">
+        <v>392</v>
+      </c>
+      <c r="C13" t="s">
+        <v>393</v>
+      </c>
+      <c r="D13" t="s">
+        <v>394</v>
+      </c>
+      <c r="E13" t="s">
+        <v>395</v>
+      </c>
+      <c r="F13" t="s">
+        <v>396</v>
+      </c>
+      <c r="G13">
+        <v>2</v>
+      </c>
+      <c r="H13">
+        <v>1</v>
+      </c>
+      <c r="I13">
+        <v>2</v>
+      </c>
+      <c r="J13">
+        <v>2</v>
+      </c>
+      <c r="K13" s="2">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="L13">
+        <v>5</v>
+      </c>
+      <c r="M13" t="s">
+        <v>390</v>
+      </c>
+      <c r="N13" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>367</v>
+      </c>
+      <c r="B14" t="s">
+        <v>397</v>
+      </c>
+      <c r="C14" t="s">
+        <v>398</v>
+      </c>
+      <c r="D14" t="s">
+        <v>399</v>
+      </c>
+      <c r="E14" t="s">
+        <v>400</v>
+      </c>
+      <c r="F14" t="s">
+        <v>401</v>
+      </c>
+      <c r="G14">
+        <v>1</v>
+      </c>
+      <c r="H14">
+        <v>1</v>
+      </c>
+      <c r="I14">
+        <v>1</v>
+      </c>
+      <c r="J14">
+        <v>2</v>
+      </c>
+      <c r="K14" s="2">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="L14">
+        <v>10</v>
+      </c>
+      <c r="M14" t="s">
+        <v>390</v>
+      </c>
+      <c r="N14" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="24" spans="11:11" x14ac:dyDescent="0.2">
+      <c r="K24" s="2"/>
+    </row>
+    <row r="25" spans="11:11" x14ac:dyDescent="0.2">
+      <c r="K25" s="2"/>
+    </row>
+    <row r="26" spans="11:11" x14ac:dyDescent="0.2">
+      <c r="K26" s="2"/>
+    </row>
+    <row r="27" spans="11:11" x14ac:dyDescent="0.2">
+      <c r="K27" s="2"/>
+    </row>
+    <row r="28" spans="11:11" x14ac:dyDescent="0.2">
+      <c r="K28" s="2"/>
+    </row>
+    <row r="29" spans="11:11" x14ac:dyDescent="0.2">
+      <c r="K29" s="2"/>
+    </row>
+    <row r="30" spans="11:11" x14ac:dyDescent="0.2">
+      <c r="K30" s="2"/>
+    </row>
+    <row r="31" spans="11:11" x14ac:dyDescent="0.2">
+      <c r="K31" s="2"/>
+    </row>
+    <row r="32" spans="11:11" x14ac:dyDescent="0.2">
+      <c r="K32" s="2"/>
+    </row>
+    <row r="33" spans="11:11" x14ac:dyDescent="0.2">
+      <c r="K33" s="2"/>
+    </row>
+    <row r="34" spans="11:11" x14ac:dyDescent="0.2">
+      <c r="K34" s="2"/>
+    </row>
+    <row r="35" spans="11:11" x14ac:dyDescent="0.2">
+      <c r="K35" s="2"/>
+    </row>
+    <row r="36" spans="11:11" x14ac:dyDescent="0.2">
+      <c r="K36" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>

<commit_message>
07: write-up draft, hand check
</commit_message>
<xml_diff>
--- a/model.xlsx
+++ b/model.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nasir/dev/rizm-fve-takehome-henkel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{332CFEF8-766C-1244-98CB-F3FC613E6600}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9EE0864-56CF-B740-AA25-1BA9688B4EC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21660" activeTab="3" xr2:uid="{D8DCC835-E62D-D344-B61D-C7363F95AE03}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21660" activeTab="4" xr2:uid="{D8DCC835-E62D-D344-B61D-C7363F95AE03}"/>
   </bookViews>
   <sheets>
     <sheet name="sources" sheetId="4" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1328" uniqueCount="786">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1456" uniqueCount="835">
   <si>
     <t>id</t>
   </si>
@@ -2401,6 +2401,153 @@
   </si>
   <si>
     <t>the bracket of row 62 set to zero and solved for v_h, my rearrangement of the thread's formula: v_be = c_f / η_GT − q × c_f / η_B; the GT pays in every hour with power worth more than this</t>
+  </si>
+  <si>
+    <t>what</t>
+  </si>
+  <si>
+    <t>remark</t>
+  </si>
+  <si>
+    <t>EUR/MWh</t>
+  </si>
+  <si>
+    <t>sigma</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>phi</t>
+  </si>
+  <si>
+    <t>dm</t>
+  </si>
+  <si>
+    <t>EUR/a</t>
+  </si>
+  <si>
+    <t>kappa</t>
+  </si>
+  <si>
+    <t>(188994+34824)/0.0249</t>
+  </si>
+  <si>
+    <t>c_f*F*sigma</t>
+  </si>
+  <si>
+    <t>57.8*1050000*0.015</t>
+  </si>
+  <si>
+    <t>Q_dh*phi*dm</t>
+  </si>
+  <si>
+    <t>30000*0.2*60</t>
+  </si>
+  <si>
+    <t>kappa*(fuel+heat)-O1</t>
+  </si>
+  <si>
+    <t>t/a</t>
+  </si>
+  <si>
+    <t>S1/T</t>
+  </si>
+  <si>
+    <t>EUR/t</t>
+  </si>
+  <si>
+    <t>diff calc D29</t>
+  </si>
+  <si>
+    <t>should be 0</t>
+  </si>
+  <si>
+    <t>diff calc D31</t>
+  </si>
+  <si>
+    <t>should be ~0, T_group rounded</t>
+  </si>
+  <si>
+    <t>P_GT</t>
+  </si>
+  <si>
+    <t>eta_GT</t>
+  </si>
+  <si>
+    <t>h_GT</t>
+  </si>
+  <si>
+    <t>h/a</t>
+  </si>
+  <si>
+    <t>MWh/a</t>
+  </si>
+  <si>
+    <t>8.6/0.3*6000</t>
+  </si>
+  <si>
+    <t>F-F_GT</t>
+  </si>
+  <si>
+    <t>kappa*c_f*F_B*s11-O11</t>
+  </si>
+  <si>
+    <t>S11/T</t>
+  </si>
+  <si>
+    <t>T from row 16</t>
+  </si>
+  <si>
+    <t>diff calc D54</t>
+  </si>
+  <si>
+    <t>diff calc D56</t>
+  </si>
+  <si>
+    <t>should be ~0</t>
+  </si>
+  <si>
+    <t>cross checks</t>
+  </si>
+  <si>
+    <t>VET 2025</t>
+  </si>
+  <si>
+    <t>scope1 own</t>
+  </si>
+  <si>
+    <t>scope1 3rd party</t>
+  </si>
+  <si>
+    <t>plant / group gross scope1</t>
+  </si>
+  <si>
+    <t>59 %, matches R16 order of magnitude</t>
+  </si>
+  <si>
+    <t>own generation</t>
+  </si>
+  <si>
+    <t>eta plant</t>
+  </si>
+  <si>
+    <t>fuel implied</t>
+  </si>
+  <si>
+    <t>gen/eta</t>
+  </si>
+  <si>
+    <t>implied / F</t>
+  </si>
+  <si>
+    <t>4 % over F, ok (red team #9)</t>
+  </si>
+  <si>
+    <t>ok</t>
+  </si>
+  <si>
+    <t>hand check 2025-09-27, values typed from assumptions, no links (except the diff cells at the end)</t>
   </si>
 </sst>
 </file>
@@ -2455,10 +2602,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -2833,23 +2979,23 @@
     <col min="6" max="6" width="44.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>250</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="3" t="s">
         <v>4</v>
       </c>
     </row>
@@ -3315,50 +3461,50 @@
     <col min="15" max="15" width="13.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="K1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="M1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="N1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="O1" s="3" t="s">
         <v>16</v>
       </c>
     </row>
@@ -5099,7 +5245,7 @@
       <c r="B43" t="s">
         <v>543</v>
       </c>
-      <c r="C43" s="2" t="s">
+      <c r="C43" t="s">
         <v>544</v>
       </c>
       <c r="D43">
@@ -6274,47 +6420,47 @@
     <col min="13" max="13" width="7.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:14" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="K1" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="M1" s="3" t="s">
         <v>403</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="N1" s="3" t="s">
         <v>309</v>
       </c>
     </row>
@@ -6900,31 +7046,31 @@
     <col min="6" max="6" width="9.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
         <v>408</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>620</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>409</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>410</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="3" t="s">
         <v>411</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="3" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>412</v>
       </c>
     </row>
@@ -7244,12 +7390,12 @@
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="3" t="s">
         <v>441</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="3" t="s">
         <v>763</v>
       </c>
       <c r="G20" t="s">
@@ -7371,7 +7517,7 @@
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A26" s="2" t="s">
+      <c r="A26" t="s">
         <v>453</v>
       </c>
       <c r="B26" t="s">
@@ -7446,7 +7592,7 @@
       <c r="C29" t="s">
         <v>376</v>
       </c>
-      <c r="D29" s="5">
+      <c r="D29" s="4">
         <f>D28*(D21*D22*D23+D24*D25*D26)-D27</f>
         <v>1070350</v>
       </c>
@@ -7482,7 +7628,7 @@
       <c r="C31" t="s">
         <v>439</v>
       </c>
-      <c r="D31" s="6">
+      <c r="D31" s="5">
         <f>D29/D30</f>
         <v>1.1907762110286035</v>
       </c>
@@ -7500,7 +7646,7 @@
       <c r="C32" t="s">
         <v>439</v>
       </c>
-      <c r="D32" s="3">
+      <c r="D32" s="2">
         <f>D29/D16</f>
         <v>0.79385080735240232</v>
       </c>
@@ -7524,7 +7670,7 @@
       <c r="C33" t="s">
         <v>439</v>
       </c>
-      <c r="D33" s="3">
+      <c r="D33" s="2">
         <f>D29/D15</f>
         <v>2.3815524220572071</v>
       </c>
@@ -7719,12 +7865,12 @@
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A43" s="4" t="s">
+      <c r="A43" s="3" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A44" s="4" t="s">
+      <c r="A44" s="3" t="s">
         <v>776</v>
       </c>
       <c r="G44" t="s">
@@ -7933,7 +8079,7 @@
       <c r="C54" t="s">
         <v>376</v>
       </c>
-      <c r="D54" s="5">
+      <c r="D54" s="4">
         <f>D53*D45*D50*D51-D52</f>
         <v>407484</v>
       </c>
@@ -7966,7 +8112,7 @@
       <c r="C56" t="s">
         <v>439</v>
       </c>
-      <c r="D56" s="6">
+      <c r="D56" s="5">
         <f>D54/D55</f>
         <v>0.45333045599549632</v>
       </c>
@@ -7981,7 +8127,7 @@
       <c r="C57" t="s">
         <v>439</v>
       </c>
-      <c r="D57" s="3">
+      <c r="D57" s="2">
         <f>D54/D16</f>
         <v>0.30222030399699756</v>
       </c>
@@ -8002,7 +8148,7 @@
       <c r="C58" t="s">
         <v>439</v>
       </c>
-      <c r="D58" s="3">
+      <c r="D58" s="2">
         <f>D54/D15</f>
         <v>0.90666091199099264</v>
       </c>
@@ -8032,12 +8178,12 @@
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A61" s="4" t="s">
+      <c r="A61" s="3" t="s">
         <v>778</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A62" s="4" t="s">
+      <c r="A62" s="3" t="s">
         <v>779</v>
       </c>
       <c r="G62" t="s">
@@ -8273,7 +8419,7 @@
       <c r="C73" t="s">
         <v>443</v>
       </c>
-      <c r="D73" s="6">
+      <c r="D73" s="5">
         <f>D68/D64-D66*D68/D67</f>
         <v>90.050724637681157</v>
       </c>
@@ -8305,9 +8451,620 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8AB672FE-D8FE-194D-AD1E-1938348FC52B}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="23" customWidth="1"/>
+    <col min="2" max="2" width="4.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="32.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>834</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>786</v>
+      </c>
+      <c r="B2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>409</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>641</v>
+      </c>
+      <c r="B3" t="s">
+        <v>444</v>
+      </c>
+      <c r="C3">
+        <v>57.8</v>
+      </c>
+      <c r="D3" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>621</v>
+      </c>
+      <c r="B4" t="s">
+        <v>415</v>
+      </c>
+      <c r="C4">
+        <v>1050000</v>
+      </c>
+      <c r="D4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>789</v>
+      </c>
+      <c r="B5" t="s">
+        <v>447</v>
+      </c>
+      <c r="C5">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="D5" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>644</v>
+      </c>
+      <c r="B6" t="s">
+        <v>450</v>
+      </c>
+      <c r="C6">
+        <v>30000</v>
+      </c>
+      <c r="D6" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>791</v>
+      </c>
+      <c r="B7" t="s">
+        <v>452</v>
+      </c>
+      <c r="C7">
+        <v>0.2</v>
+      </c>
+      <c r="D7" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>792</v>
+      </c>
+      <c r="B8" t="s">
+        <v>455</v>
+      </c>
+      <c r="C8">
+        <v>60</v>
+      </c>
+      <c r="D8" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>648</v>
+      </c>
+      <c r="B9" t="s">
+        <v>457</v>
+      </c>
+      <c r="C9">
+        <v>200000</v>
+      </c>
+      <c r="D9" t="s">
+        <v>793</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>794</v>
+      </c>
+      <c r="B10" t="s">
+        <v>740</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>632</v>
+      </c>
+      <c r="B11" t="s">
+        <v>132</v>
+      </c>
+      <c r="C11">
+        <v>8988675</v>
+      </c>
+      <c r="D11" t="s">
+        <v>134</v>
+      </c>
+      <c r="E11" t="s">
+        <v>795</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>633</v>
+      </c>
+      <c r="B12" t="s">
+        <v>431</v>
+      </c>
+      <c r="C12">
+        <v>0.1</v>
+      </c>
+      <c r="D12" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>796</v>
+      </c>
+      <c r="C13">
+        <f>C3*C4*C5</f>
+        <v>910350</v>
+      </c>
+      <c r="D13" t="s">
+        <v>793</v>
+      </c>
+      <c r="E13" t="s">
+        <v>797</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>798</v>
+      </c>
+      <c r="C14">
+        <f>C6*C7*C8</f>
+        <v>360000</v>
+      </c>
+      <c r="D14" t="s">
+        <v>793</v>
+      </c>
+      <c r="E14" t="s">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15">
+        <f>C10*(C13+C14)-C9</f>
+        <v>1070350</v>
+      </c>
+      <c r="D15" t="s">
+        <v>793</v>
+      </c>
+      <c r="E15" t="s">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>634</v>
+      </c>
+      <c r="C16">
+        <f>C11*C12</f>
+        <v>898867.5</v>
+      </c>
+      <c r="D16" t="s">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>802</v>
+      </c>
+      <c r="C17">
+        <f>C15/C16</f>
+        <v>1.1907761711264453</v>
+      </c>
+      <c r="D17" t="s">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>804</v>
+      </c>
+      <c r="C18">
+        <f>calc!D29-C15</f>
+        <v>0</v>
+      </c>
+      <c r="D18" t="s">
+        <v>793</v>
+      </c>
+      <c r="E18" t="s">
+        <v>805</v>
+      </c>
+      <c r="F18" t="s">
+        <v>833</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>806</v>
+      </c>
+      <c r="C19" s="2">
+        <f>calc!D31-C17</f>
+        <v>3.99021582442316E-8</v>
+      </c>
+      <c r="D19" t="s">
+        <v>803</v>
+      </c>
+      <c r="E19" t="s">
+        <v>807</v>
+      </c>
+      <c r="F19" t="s">
+        <v>833</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>641</v>
+      </c>
+      <c r="B22" t="s">
+        <v>444</v>
+      </c>
+      <c r="C22">
+        <v>57.8</v>
+      </c>
+      <c r="D22" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>621</v>
+      </c>
+      <c r="B23" t="s">
+        <v>415</v>
+      </c>
+      <c r="C23">
+        <v>1050000</v>
+      </c>
+      <c r="D23" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>808</v>
+      </c>
+      <c r="B24" t="s">
+        <v>217</v>
+      </c>
+      <c r="C24">
+        <v>8600</v>
+      </c>
+      <c r="D24" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>809</v>
+      </c>
+      <c r="B25" t="s">
+        <v>485</v>
+      </c>
+      <c r="C25">
+        <v>0.3</v>
+      </c>
+      <c r="D25" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>810</v>
+      </c>
+      <c r="B26" t="s">
+        <v>488</v>
+      </c>
+      <c r="C26">
+        <v>6000</v>
+      </c>
+      <c r="D26" t="s">
+        <v>811</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>666</v>
+      </c>
+      <c r="B27" t="s">
+        <v>493</v>
+      </c>
+      <c r="C27">
+        <v>0.01</v>
+      </c>
+      <c r="D27" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>668</v>
+      </c>
+      <c r="B28" t="s">
+        <v>494</v>
+      </c>
+      <c r="C28">
+        <v>100000</v>
+      </c>
+      <c r="D28" t="s">
+        <v>793</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>794</v>
+      </c>
+      <c r="B29" t="s">
+        <v>740</v>
+      </c>
+      <c r="C29">
+        <v>1</v>
+      </c>
+      <c r="D29" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>662</v>
+      </c>
+      <c r="C30">
+        <f>C24/1000/C25*C26</f>
+        <v>172000</v>
+      </c>
+      <c r="D30" t="s">
+        <v>812</v>
+      </c>
+      <c r="E30" t="s">
+        <v>813</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>664</v>
+      </c>
+      <c r="C31">
+        <f>C23-C30</f>
+        <v>878000</v>
+      </c>
+      <c r="D31" t="s">
+        <v>812</v>
+      </c>
+      <c r="E31" t="s">
+        <v>814</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>267</v>
+      </c>
+      <c r="C32">
+        <f>C29*C22*C31*C27-C28</f>
+        <v>407484</v>
+      </c>
+      <c r="D32" t="s">
+        <v>793</v>
+      </c>
+      <c r="E32" t="s">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>816</v>
+      </c>
+      <c r="C33">
+        <f>C32/C16</f>
+        <v>0.45333044080467921</v>
+      </c>
+      <c r="D33" t="s">
+        <v>803</v>
+      </c>
+      <c r="E33" t="s">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>818</v>
+      </c>
+      <c r="C34">
+        <f>calc!D54-C32</f>
+        <v>0</v>
+      </c>
+      <c r="D34" t="s">
+        <v>793</v>
+      </c>
+      <c r="E34" t="s">
+        <v>805</v>
+      </c>
+      <c r="F34" t="s">
+        <v>833</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>819</v>
+      </c>
+      <c r="C35" s="2">
+        <f>calc!D56-C33</f>
+        <v>1.5190817104215881E-8</v>
+      </c>
+      <c r="D35" t="s">
+        <v>803</v>
+      </c>
+      <c r="E35" t="s">
+        <v>820</v>
+      </c>
+      <c r="F35" t="s">
+        <v>833</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>822</v>
+      </c>
+      <c r="B38" t="s">
+        <v>238</v>
+      </c>
+      <c r="C38">
+        <v>211078</v>
+      </c>
+      <c r="D38" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>823</v>
+      </c>
+      <c r="B39" t="s">
+        <v>108</v>
+      </c>
+      <c r="C39">
+        <v>188994</v>
+      </c>
+      <c r="D39" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>824</v>
+      </c>
+      <c r="B40" t="s">
+        <v>108</v>
+      </c>
+      <c r="C40">
+        <v>168856</v>
+      </c>
+      <c r="D40" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>825</v>
+      </c>
+      <c r="C41">
+        <f>C38/(C39+C40)</f>
+        <v>0.58985049601788464</v>
+      </c>
+      <c r="D41" t="s">
+        <v>790</v>
+      </c>
+      <c r="E41" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>827</v>
+      </c>
+      <c r="B42" t="s">
+        <v>101</v>
+      </c>
+      <c r="C42">
+        <v>930585</v>
+      </c>
+      <c r="D42" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>828</v>
+      </c>
+      <c r="B43" t="s">
+        <v>199</v>
+      </c>
+      <c r="C43">
+        <v>0.85</v>
+      </c>
+      <c r="D43" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>829</v>
+      </c>
+      <c r="C44">
+        <f>C42/C43</f>
+        <v>1094805.8823529412</v>
+      </c>
+      <c r="D44" t="s">
+        <v>812</v>
+      </c>
+      <c r="E44" t="s">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>831</v>
+      </c>
+      <c r="C45">
+        <f>C44/C23</f>
+        <v>1.0426722689075631</v>
+      </c>
+      <c r="D45" t="s">
+        <v>790</v>
+      </c>
+      <c r="E45" t="s">
+        <v>832</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>